<commit_message>
Set patient_starts as base-case demand mode with cohort duration logic
</commit_message>
<xml_diff>
--- a/templates/CBX250_Model_Assumptions_Template.xlsx
+++ b/templates/CBX250_Model_Assumptions_Template.xlsx
@@ -9,13 +9,14 @@
     <sheet name="Scenario_Controls" sheetId="2" r:id="rId2"/>
     <sheet name="Launch_Timing" sheetId="3" r:id="rId3"/>
     <sheet name="Dosing_Assumptions" sheetId="4" r:id="rId4"/>
-    <sheet name="Product_Parameters" sheetId="5" r:id="rId5"/>
-    <sheet name="Yield_Assumptions" sheetId="6" r:id="rId6"/>
-    <sheet name="Packaging_and_Vialing" sheetId="7" r:id="rId7"/>
-    <sheet name="SS_Assumptions" sheetId="8" r:id="rId8"/>
-    <sheet name="CML_Prevalent_Assumptions" sheetId="9" r:id="rId9"/>
-    <sheet name="Trade_Inventory_FutureHooks" sheetId="10" r:id="rId10"/>
-    <sheet name="Lookup_Lists" sheetId="11" r:id="rId11"/>
+    <sheet name="Treatment_Duration_Assumptions" sheetId="5" r:id="rId5"/>
+    <sheet name="Product_Parameters" sheetId="6" r:id="rId6"/>
+    <sheet name="Yield_Assumptions" sheetId="7" r:id="rId7"/>
+    <sheet name="Packaging_and_Vialing" sheetId="8" r:id="rId8"/>
+    <sheet name="SS_Assumptions" sheetId="9" r:id="rId9"/>
+    <sheet name="CML_Prevalent_Assumptions" sheetId="10" r:id="rId10"/>
+    <sheet name="Trade_Inventory_FutureHooks" sheetId="11" r:id="rId11"/>
+    <sheet name="Lookup_Lists" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -131,7 +132,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -203,90 +204,107 @@
       </c>
       <c r="C4" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">One active Scenario_Controls row is required. Dosing_Assumptions should provide one active module row for AML, MDS, CML_Incident, and CML_Prevalent.</t>
+          <t xml:space="preserve">One active Scenario_Controls row is required. Dosing_Assumptions should provide one active module row for AML, MDS, CML_Incident, and CML_Prevalent. The seeded base case uses demand_basis = patient_starts, so populate active Treatment_Duration_Assumptions rows before running the forecast workflow.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Scope precedence</t>
+          <t xml:space="preserve">Phase 1 demand basis</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">When a sheet supports both scenario-level defaults and module-specific overrides, module-specific override rows take precedence over scenario-default rows.</t>
+          <t xml:space="preserve">patient_starts is the preferred default operating mode and represents the approved base-case commercial input path.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Current generated Phase 2 config already applies this precedence for module FG mg per unit. For ds_qty_per_dp_unit_mg and ds_overage_factor, module overrides are preserved in normalized artifacts but the current engine still consumes the scenario default only.</t>
+          <t xml:space="preserve">treated_census remains supported for backward compatibility and special cases only. Do not apply duration logic on top of already treated-census inputs.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Current engine wiring</t>
+          <t xml:space="preserve">Scope precedence</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">The importer generates machine-readable CSV artifacts plus generated_phase2_parameters.toml and generated_phase2_scenario.toml.</t>
+          <t xml:space="preserve">When a sheet supports both scenario-level defaults and module-specific overrides, module-specific override rows take precedence over scenario-default rows.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Current Phase 2 wiring consumes: dose_basis_default, module-specific dosing values, module FG mg per unit, module FG vialing rule, global yields, DS quantity per DP unit default, DS overage default, SS ratio, and co_pack_mode.</t>
+          <t xml:space="preserve">Current generated Phase 2 config already applies this precedence for module FG mg per unit. For ds_qty_per_dp_unit_mg and ds_overage_factor, module overrides are preserved in normalized artifacts but the current engine still consumes the scenario default only.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Future-ready fields</t>
+          <t xml:space="preserve">Current engine wiring</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Launch_Timing, geography-specific overrides, segment-specific overrides, dp_concentration_mg_per_ml, dp_fill_volume_ml, and Trade_Inventory_FutureHooks are preserved in normalized outputs even if not yet wired into active model logic.</t>
+          <t xml:space="preserve">The importer generates machine-readable CSV artifacts plus generated_phase2_parameters.toml and generated_phase2_scenario.toml.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">CML_Prevalent_Assumptions remains a dedicated artifact sheet. Populate approved pool, timing, and exhaustion metadata here without treating CML like AML/MDS segment mix logic.</t>
+          <t xml:space="preserve">Current wiring consumes: Scenario_Controls.demand_basis plus Treatment_Duration_Assumptions for Phase 1 starts-based mode, and dose_basis_default, module-specific dosing values, module FG mg per unit, module FG vialing rule, global yields, DS quantity per DP unit default, DS overage default, SS ratio, and co_pack_mode for Phase 2.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Workbook to model bridge</t>
+          <t xml:space="preserve">Future-ready fields</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">After import, use the generated Phase 2 scenario directly or pass it into the one-command forecast workflow as --phase2-scenario.</t>
+          <t xml:space="preserve">Launch_Timing, geography-specific overrides, segment-specific overrides, dp_concentration_mg_per_ml, dp_fill_volume_ml, and Trade_Inventory_FutureHooks are preserved in normalized outputs even if not yet wired into active model logic.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">This keeps the current architecture intact while removing the need to edit TOML by hand for the active deterministic assumptions.</t>
+          <t xml:space="preserve">CML_Prevalent_Assumptions remains a dedicated artifact sheet. Populate approved pool, timing, and exhaustion metadata here without treating CML like AML/MDS segment mix logic.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="4">
         <is>
+          <t xml:space="preserve">Workbook to model bridge</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="8">
+        <is>
+          <t xml:space="preserve">After import, use the generated Phase 2 scenario directly or pass the assumptions workbook into the one-command forecast workflow.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="8">
+        <is>
+          <t xml:space="preserve">This keeps the current architecture intact while removing the need to edit TOML by hand for the active deterministic assumptions. The workflow also consumes the generated treatment duration artifact when demand_basis = patient_starts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="4">
+        <is>
           <t xml:space="preserve">Approved base-case defaults</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="8">
-        <is>
-          <t xml:space="preserve">Seeded defaults reflect the current approved Phase 2 base case: fixed dose 0.15 mg, weight-based 0.0023 mg/kg, deterministic average weight 80 kg, AML/MDS 4.33 doses per month, CML modules 1.00 dose per month, fg_mg_per_unit 1.0 mg, DS quantity per DP unit 1.0 mg, ds_to_dp_yield 0.90, dp_to_fg_yield 0.98, ds_overage_factor 0.05, ss_ratio_to_fg 1.0.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr" s="8">
+      <c r="B10" t="inlineStr" s="8">
+        <is>
+          <t xml:space="preserve">Seeded defaults reflect the current approved base case: annual patient_starts for Phase 1, fixed dose 0.15 mg, weight-based 0.0023 mg/kg, deterministic average weight 80 kg, AML/MDS 4.33 doses per month, CML modules 1.00 dose per month, fg_mg_per_unit 1.0 mg, DS quantity per DP unit 1.0 mg, ds_to_dp_yield 0.90, dp_to_fg_yield 0.98, ds_overage_factor 0.05, ss_ratio_to_fg 1.0.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Where the approved contract is still unresolved, rows are labeled PLACEHOLDER rather than silently inventing a final business assumption.</t>
         </is>
@@ -299,6 +317,829 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:N41"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="72" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">scenario_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">geography_code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">addressable_prevalent_pool</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">launch_year_index</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">launch_month_index</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">duration_months</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">curve_profile_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">bolus_start_year</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">bolus_end_year</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">exhaustion_year</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">exhaustion_rule</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">source</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">active_flag</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">US</t>
+        </is>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2">
+        <v>12</v>
+      </c>
+      <c r="G2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PLACEHOLDER_PROFILE</t>
+        </is>
+      </c>
+      <c r="H2" s="2">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2">
+        <v>3</v>
+      </c>
+      <c r="J2" s="2">
+        <v>4</v>
+      </c>
+      <c r="K2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">track_vs_pool</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">PLACEHOLDER populate approved US prevalent pool inputs before activating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">EU</t>
+        </is>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2">
+        <v>12</v>
+      </c>
+      <c r="G3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PLACEHOLDER_PROFILE</t>
+        </is>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2">
+        <v>3</v>
+      </c>
+      <c r="J3" s="2">
+        <v>4</v>
+      </c>
+      <c r="K3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">track_vs_pool</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">PLACEHOLDER populate approved EU prevalent pool inputs before activating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="9"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="9"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="9"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="9"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="9"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="9"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="9"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="9"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="9"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="9"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="9"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="9"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="9"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="9"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="9"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="9"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="9"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="9"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="9"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="9"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="9"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="9"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="9"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="9"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="9"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
+      <c r="L29" s="2"/>
+      <c r="M29" s="2"/>
+      <c r="N29" s="9"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="9"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="9"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="9"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
+      <c r="N33" s="9"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+      <c r="N34" s="9"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="9"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="9"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
+      <c r="N37" s="9"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+      <c r="N38" s="9"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
+      <c r="N39" s="9"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+      <c r="M40" s="2"/>
+      <c r="N40" s="9"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+      <c r="M41" s="2"/>
+      <c r="N41" s="9"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N1"/>
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="K2:K41" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$N$2:$N$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="M2:M41" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -559,31 +1400,32 @@
   <autoFilter ref="A1:G1"/>
   <dataValidations count="1">
     <dataValidation type="list" sqref="F2:F21" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -604,50 +1446,55 @@
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">demand_basis</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">yes_no</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">true_false</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">parameter_scope</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">vialing_rule</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">co_pack_mode</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">active_flag</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">forecast_grain</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="L1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">forecast_frequency</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">partial_pack_handling</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="N1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">exhaustion_rule</t>
         </is>
@@ -671,50 +1518,55 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t xml:space="preserve">patient_starts</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t xml:space="preserve">true</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t xml:space="preserve">scenario_default</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t xml:space="preserve">patient_dose_ceiling</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t xml:space="preserve">separate_sku_first</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t xml:space="preserve">module_level</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">monthly</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t xml:space="preserve">annual</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t xml:space="preserve">full_pack_consumed</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">track_vs_pool</t>
         </is>
@@ -738,50 +1590,55 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t xml:space="preserve">treated_census</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t xml:space="preserve">no</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t xml:space="preserve">false</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t xml:space="preserve">module_override</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">segment_level</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">annual</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t xml:space="preserve">monthly</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">placeholder_metadata_only</t>
         </is>
@@ -850,6 +1707,11 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t xml:space="preserve">validate_only</t>
         </is>
       </c>
@@ -920,6 +1782,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -987,6 +1854,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1054,16 +1926,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1"/>
+  <autoFilter ref="A1:N1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1072,8 +1949,9 @@
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="56" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="56" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1104,15 +1982,20 @@
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">demand_basis</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">dose_basis_default</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">base_currency</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">notes</t>
         </is>
@@ -1141,22 +2024,27 @@
       </c>
       <c r="E2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">monthly</t>
+          <t xml:space="preserve">annual</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">patient_starts</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">fixed</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="2">
+      <c r="H2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">USD</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">Edit this row instead of hand-editing Phase 2 TOML files.</t>
+      <c r="I2" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Edit this row instead of hand-editing config files. Seeded for the annual patient_starts base case.</t>
         </is>
       </c>
     </row>
@@ -1168,7 +2056,8 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="9"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="9"/>
     </row>
     <row r="4">
       <c r="A4" s="2"/>
@@ -1178,7 +2067,8 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="9"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="9"/>
     </row>
     <row r="5">
       <c r="A5" s="2"/>
@@ -1188,7 +2078,8 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="9"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="9"/>
     </row>
     <row r="6">
       <c r="A6" s="2"/>
@@ -1198,7 +2089,8 @@
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="9"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="9"/>
     </row>
     <row r="7">
       <c r="A7" s="2"/>
@@ -1208,7 +2100,8 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="9"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="9"/>
     </row>
     <row r="8">
       <c r="A8" s="2"/>
@@ -1218,7 +2111,8 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="9"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="9"/>
     </row>
     <row r="9">
       <c r="A9" s="2"/>
@@ -1228,7 +2122,8 @@
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="9"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="9"/>
     </row>
     <row r="10">
       <c r="A10" s="2"/>
@@ -1238,7 +2133,8 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
-      <c r="H10" s="9"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="9"/>
     </row>
     <row r="11">
       <c r="A11" s="2"/>
@@ -1248,21 +2144,25 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="9"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
-  <dataValidations count="4">
+  <autoFilter ref="A1:I1"/>
+  <dataValidations count="5">
     <dataValidation type="list" sqref="C2:C11" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="D2:D11" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
+      <formula1>Lookup_Lists!$K$2:$K$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="E2:E11" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$K$2:$K$3</formula1>
+      <formula1>Lookup_Lists!$L$2:$L$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F2:F11" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$D$2:$D$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="G2:G11" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$C$2:$C$3</formula1>
     </dataValidation>
   </dataValidations>
@@ -1776,7 +2676,7 @@
       <formula1>Lookup_Lists!$A$2:$A$5</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F2:F41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3632,13 +4532,13 @@
       <formula1>Lookup_Lists!$C$2:$C$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="J2:J81" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$E$2:$E$3</formula1>
+      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="L2:L81" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$E$2:$E$3</formula1>
+      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="P2:P81" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3646,6 +4546,599 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G41"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="72" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">scenario_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">module</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">segment_code</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">geography_code</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">treatment_duration_months</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">active_flag</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AML</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1L_fit</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="E2" s="2">
+        <v>12</v>
+      </c>
+      <c r="F2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved base-case duration default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AML</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1L_unfit</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="E3" s="2">
+        <v>10</v>
+      </c>
+      <c r="F3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved base-case duration default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AML</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">RR</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="E4" s="2">
+        <v>6</v>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved base-case duration default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MDS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">HR_MDS</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="E5" s="2">
+        <v>12</v>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved base-case duration default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MDS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LR_MDS</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="E6" s="2">
+        <v>12</v>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved base-case duration default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CML_Incident</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CML_Incident</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="E7" s="2">
+        <v>24</v>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved base-case duration default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CML_Prevalent</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CML_Prevalent</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="E8" s="2">
+        <v>24</v>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved base-case duration default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="9"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="9"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="9"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="9"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="9"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="9"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="9"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="9"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="9"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="9"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="9"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="9"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="9"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="9"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="9"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1"/>
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="B2:B41" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$A$2:$A$5</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="F2:F41" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J41"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -4250,20 +5743,20 @@
   <autoFilter ref="A1:J1"/>
   <dataValidations count="3">
     <dataValidation type="list" sqref="B2:B41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
+      <formula1>Lookup_Lists!$G$2:$G$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="C2:C41" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$B$2:$B$6</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I2:I41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:K41"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -4926,20 +6419,20 @@
   <autoFilter ref="A1:K1"/>
   <dataValidations count="3">
     <dataValidation type="list" sqref="B2:B41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
+      <formula1>Lookup_Lists!$G$2:$G$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="C2:C41" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$B$2:$B$6</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="J2:J41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J41"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -5639,23 +7132,23 @@
       <formula1>Lookup_Lists!$A$2:$A$5</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="D2:D41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$G$2:$G$2</formula1>
+      <formula1>Lookup_Lists!$H$2:$H$2</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="E2:F41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$E$2:$E$3</formula1>
+      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="H2:H41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$L$2:$L$2</formula1>
+      <formula1>Lookup_Lists!$M$2:$M$2</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I2:I41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -5917,833 +7410,10 @@
       <formula1>Lookup_Lists!$B$2:$B$6</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="E2:E21" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$H$2:$H$2</formula1>
+      <formula1>Lookup_Lists!$I$2:$I$2</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F2:F21" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N41"/>
-  <sheetFormatPr defaultRowHeight="18"/>
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="72" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">scenario_name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">geography_code</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">addressable_prevalent_pool</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">launch_year_index</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">launch_month_index</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">duration_months</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">curve_profile_id</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">bolus_start_year</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">bolus_end_year</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">exhaustion_year</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">exhaustion_rule</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">source</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">active_flag</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3">
-        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
-      </c>
-      <c r="B2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">US</t>
-        </is>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2">
-        <v>12</v>
-      </c>
-      <c r="G2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">PLACEHOLDER_PROFILE</t>
-        </is>
-      </c>
-      <c r="H2" s="2">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2">
-        <v>3</v>
-      </c>
-      <c r="J2" s="2">
-        <v>4</v>
-      </c>
-      <c r="K2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">track_vs_pool</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">PLACEHOLDER</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">PLACEHOLDER populate approved US prevalent pool inputs before activating.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3">
-        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
-      </c>
-      <c r="B3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">EU</t>
-        </is>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2">
-        <v>1</v>
-      </c>
-      <c r="F3" s="2">
-        <v>12</v>
-      </c>
-      <c r="G3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">PLACEHOLDER_PROFILE</t>
-        </is>
-      </c>
-      <c r="H3" s="2">
-        <v>1</v>
-      </c>
-      <c r="I3" s="2">
-        <v>3</v>
-      </c>
-      <c r="J3" s="2">
-        <v>4</v>
-      </c>
-      <c r="K3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">track_vs_pool</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">PLACEHOLDER</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">PLACEHOLDER populate approved EU prevalent pool inputs before activating.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="9"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="9"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="9"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="9"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="9"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="9"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="9"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="9"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="9"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="9"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="9"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="9"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="9"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="9"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="9"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="9"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="9"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="9"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="9"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="9"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="9"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="9"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="9"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
-      <c r="N27" s="9"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-      <c r="N28" s="9"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="9"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="9"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="9"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="9"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="9"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
-      <c r="N34" s="9"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
-      <c r="N35" s="9"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-      <c r="N36" s="9"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="3"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="9"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="3"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-      <c r="N38" s="9"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
-      <c r="K39" s="2"/>
-      <c r="L39" s="2"/>
-      <c r="M39" s="2"/>
-      <c r="N39" s="9"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="3"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-      <c r="N40" s="9"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="3"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
-      <c r="N41" s="9"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:N1"/>
-  <dataValidations count="2">
-    <dataValidation type="list" sqref="K2:K41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$M$2:$M$4</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="M2:M41" showErrorMessage="1" allowBlank="1">
-      <formula1>Lookup_Lists!$I$2:$I$3</formula1>
+      <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Wire Phase 3 assumptions workbook and one-command workflow through trade layer
</commit_message>
<xml_diff>
--- a/templates/CBX250_Model_Assumptions_Template.xlsx
+++ b/templates/CBX250_Model_Assumptions_Template.xlsx
@@ -170,7 +170,7 @@
       </c>
       <c r="C2" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Users should edit Excel assumptions here rather than hand-editing TOML files. The importer converts these rows into normalized artifacts plus a generated Phase 2 parameter config.</t>
+          <t xml:space="preserve">Users should edit Excel assumptions here rather than hand-editing TOML files. The importer converts these rows into normalized artifacts plus generated Phase 2 and Phase 3 parameter configs.</t>
         </is>
       </c>
     </row>
@@ -182,12 +182,12 @@
       </c>
       <c r="B3" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Current scope covers Phase 1 and Phase 2 relevant assumptions only.</t>
+          <t xml:space="preserve">Current scope covers Phase 1, Phase 2, and the active deterministic Phase 3 trade layer assumptions.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Trade, inventory, production scheduling, financials, Monte Carlo, and UI remain later-phase work. FutureHooks rows are preserved but not wired into active logic.</t>
+          <t xml:space="preserve">Production scheduling, inventory, financials, Monte Carlo, and UI remain later-phase work. Trade_Inventory_FutureHooks now wires the active deterministic Phase 3 trade config, but broader future-phase inventory behavior remains deferred.</t>
         </is>
       </c>
     </row>
@@ -250,12 +250,12 @@
       </c>
       <c r="B7" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">The importer generates machine-readable CSV artifacts plus generated_phase2_parameters.toml and generated_phase2_scenario.toml.</t>
+          <t xml:space="preserve">The importer generates machine-readable CSV artifacts plus generated_phase2_parameters.toml / generated_phase2_scenario.toml and generated_phase3_parameters.toml / generated_phase3_scenario.toml.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Current wiring consumes: Scenario_Controls.demand_basis plus Treatment_Duration_Assumptions for Phase 1 starts-based mode, and dose_basis_default, module-specific dosing values, module FG mg per unit, module FG vialing rule, global yields, DS quantity per DP unit default, DS overage default, SS ratio, and co_pack_mode for Phase 2.</t>
+          <t xml:space="preserve">Current wiring consumes: Scenario_Controls.demand_basis plus Treatment_Duration_Assumptions for Phase 1 starts-based mode; dose_basis_default, module-specific dosing values, module FG mg per unit, module FG vialing rule, global yields, DS quantity per DP unit default, DS overage default, SS ratio, and co_pack_mode for Phase 2; and active deterministic trade parameters from Trade_Inventory_FutureHooks for Phase 3.</t>
         </is>
       </c>
     </row>
@@ -267,12 +267,12 @@
       </c>
       <c r="B8" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Launch_Timing, geography-specific overrides, segment-specific overrides, dp_concentration_mg_per_ml, dp_fill_volume_ml, and Trade_Inventory_FutureHooks are preserved in normalized outputs even if not yet wired into active model logic.</t>
+          <t xml:space="preserve">Launch_Timing, geography-specific overrides, segment-specific overrides, dp_concentration_mg_per_ml, and dp_fill_volume_ml are preserved in normalized outputs even if not yet wired into active model logic.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">CML_Prevalent_Assumptions remains a dedicated artifact sheet. Populate approved pool, timing, and exhaustion metadata here without treating CML like AML/MDS segment mix logic.</t>
+          <t xml:space="preserve">CML_Prevalent_Assumptions remains a dedicated artifact sheet. Populate approved pool, timing, and exhaustion metadata here without treating CML like AML/MDS segment mix logic. Trade_Inventory_FutureHooks still carries a historical name, but it now also feeds the active deterministic Phase 3 trade config.</t>
         </is>
       </c>
     </row>
@@ -284,12 +284,12 @@
       </c>
       <c r="B9" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">After import, use the generated Phase 2 scenario directly or pass the assumptions workbook into the one-command forecast workflow.</t>
+          <t xml:space="preserve">After import, use the generated Phase 2 or Phase 3 scenario directly, or pass the assumptions workbook into the one-command forecast workflow.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">This keeps the current architecture intact while removing the need to edit TOML by hand for the active deterministic assumptions. The workflow also consumes the generated treatment duration artifact when demand_basis = patient_starts.</t>
+          <t xml:space="preserve">This keeps the current architecture intact while removing the need to edit TOML by hand for the active deterministic assumptions. The workflow also consumes the generated treatment duration artifact when demand_basis = patient_starts and can optionally run through Phase 3.</t>
         </is>
       </c>
     </row>
@@ -1141,16 +1141,32 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="32" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="68" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="12" customWidth="1"/>
+    <col min="23" max="23" width="72" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1161,30 +1177,110 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">trade_row_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">module</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">geography_code</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">trade_rule_placeholder</t>
-        </is>
-      </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">inventory_rule_placeholder</t>
+          <t xml:space="preserve">sublayer1_target_weeks_on_hand</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">sublayer2_target_weeks_on_hand</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">sublayer2_wastage_rate</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">initial_stocking_units_per_new_site</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ss_units_per_new_site</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">sublayer1_launch_fill_months_of_demand</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">rems_certification_lag_weeks</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">january_softening_enabled</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">january_softening_factor</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">bullwhip_flag_threshold</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">channel_fill_start_prelaunch_weeks</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">sublayer2_fill_distribution_weeks</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">weeks_per_month</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">site_activation_rate</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">certified_sites_at_launch</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">certified_sites_at_peak</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">launch_month_index</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">active_flag</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="W1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">notes</t>
         </is>
@@ -1196,124 +1292,572 @@
       </c>
       <c r="B2" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">scenario_default</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">ALL</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="D2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">ALL</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">PLACEHOLDER_FUTURE_PHASE</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">PLACEHOLDER_FUTURE_PHASE</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">Future-phase placeholders only. Not wired into active model logic.</t>
+      <c r="E2" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
+        <v>6</v>
+      </c>
+      <c r="I2" s="2">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="M2" s="2">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="O2" s="2">
+        <v>4</v>
+      </c>
+      <c r="P2" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>4.33</v>
+      </c>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved deterministic Phase 3 scenario defaults. Edit here instead of phase3_trade_layer.toml.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="A3" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">geography_default</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">US</t>
+        </is>
+      </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="9"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2">
+        <v>5</v>
+      </c>
+      <c r="S3" s="2">
+        <v>5</v>
+      </c>
+      <c r="T3" s="2">
+        <v>25</v>
+      </c>
+      <c r="U3" s="2"/>
+      <c r="V3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample US site activation defaults for the deterministic Phase 3 trade layer.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="A4" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">geography_default</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">EU</t>
+        </is>
+      </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
-      <c r="G4" s="9"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2">
+        <v>3</v>
+      </c>
+      <c r="S4" s="2">
+        <v>3</v>
+      </c>
+      <c r="T4" s="2">
+        <v>18</v>
+      </c>
+      <c r="U4" s="2"/>
+      <c r="V4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample EU site activation defaults for the deterministic Phase 3 trade layer.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="A5" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AML</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">US</t>
+        </is>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
-      <c r="G5" s="9"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2">
+        <v>1</v>
+      </c>
+      <c r="V5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample launch event.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+      <c r="A6" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MDS</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">US</t>
+        </is>
+      </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="9"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2">
+        <v>1</v>
+      </c>
+      <c r="V6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample launch event.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="A7" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CML_Incident</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">US</t>
+        </is>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
-      <c r="G7" s="9"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2">
+        <v>1</v>
+      </c>
+      <c r="V7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample launch event.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="A8" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CML_Prevalent</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">US</t>
+        </is>
+      </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
-      <c r="G8" s="9"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2">
+        <v>1</v>
+      </c>
+      <c r="V8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample launch event.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
+      <c r="A9" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AML</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">EU</t>
+        </is>
+      </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
-      <c r="G9" s="9"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2">
+        <v>1</v>
+      </c>
+      <c r="V9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample launch event.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+      <c r="A10" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MDS</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">EU</t>
+        </is>
+      </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
-      <c r="G10" s="9"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+      <c r="U10" s="2">
+        <v>1</v>
+      </c>
+      <c r="V10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample launch event.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
+      <c r="A11" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CML_Incident</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">EU</t>
+        </is>
+      </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
-      <c r="G11" s="9"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2">
+        <v>1</v>
+      </c>
+      <c r="V11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample launch event.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="A12" s="3">
+        <f>IF(Scenario_Controls!$A$2="","",Scenario_Controls!$A$2)</f>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CML_Prevalent</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">EU</t>
+        </is>
+      </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
-      <c r="G12" s="9"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2">
+        <v>1</v>
+      </c>
+      <c r="V12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Approved/sample launch event.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3"/>
@@ -1322,7 +1866,23 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
-      <c r="G13" s="9"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="2"/>
+      <c r="T13" s="2"/>
+      <c r="U13" s="2"/>
+      <c r="V13" s="2"/>
+      <c r="W13" s="9"/>
     </row>
     <row r="14">
       <c r="A14" s="3"/>
@@ -1331,7 +1891,23 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="9"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
+      <c r="T14" s="2"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="2"/>
+      <c r="W14" s="9"/>
     </row>
     <row r="15">
       <c r="A15" s="3"/>
@@ -1340,7 +1916,23 @@
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="9"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+      <c r="U15" s="2"/>
+      <c r="V15" s="2"/>
+      <c r="W15" s="9"/>
     </row>
     <row r="16">
       <c r="A16" s="3"/>
@@ -1349,7 +1941,23 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="9"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
+      <c r="V16" s="2"/>
+      <c r="W16" s="9"/>
     </row>
     <row r="17">
       <c r="A17" s="3"/>
@@ -1358,7 +1966,23 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="9"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
+      <c r="V17" s="2"/>
+      <c r="W17" s="9"/>
     </row>
     <row r="18">
       <c r="A18" s="3"/>
@@ -1367,7 +1991,23 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="9"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="2"/>
+      <c r="W18" s="9"/>
     </row>
     <row r="19">
       <c r="A19" s="3"/>
@@ -1376,7 +2016,23 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-      <c r="G19" s="9"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
+      <c r="U19" s="2"/>
+      <c r="V19" s="2"/>
+      <c r="W19" s="9"/>
     </row>
     <row r="20">
       <c r="A20" s="3"/>
@@ -1385,7 +2041,23 @@
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
-      <c r="G20" s="9"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="2"/>
+      <c r="T20" s="2"/>
+      <c r="U20" s="2"/>
+      <c r="V20" s="2"/>
+      <c r="W20" s="9"/>
     </row>
     <row r="21">
       <c r="A21" s="3"/>
@@ -1394,12 +2066,37 @@
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="9"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
+      <c r="T21" s="2"/>
+      <c r="U21" s="2"/>
+      <c r="V21" s="2"/>
+      <c r="W21" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="F2:F21" showErrorMessage="1" allowBlank="1">
+  <autoFilter ref="A1:W1"/>
+  <dataValidations count="4">
+    <dataValidation type="list" sqref="B2:B21" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$O$2:$O$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="C2:C21" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$B$2:$B$6</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="L2:L21" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="V2:V21" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>
@@ -1409,7 +2106,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1426,6 +2123,7 @@
     <col min="12" max="12" width="18" customWidth="1"/>
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="14" width="24" customWidth="1"/>
+    <col min="15" max="15" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1499,6 +2197,11 @@
           <t xml:space="preserve">exhaustion_rule</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">trade_row_type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1571,6 +2274,11 @@
           <t xml:space="preserve">track_vs_pool</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scenario_default</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1643,6 +2351,11 @@
           <t xml:space="preserve">placeholder_metadata_only</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">geography_default</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1715,6 +2428,11 @@
           <t xml:space="preserve">validate_only</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">launch_event</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1787,6 +2505,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1859,6 +2582,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1931,9 +2659,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:O1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Wire Phase 4 and Phase 5 assumptions into workbook and workflow
</commit_message>
<xml_diff>
--- a/templates/CBX250_Model_Assumptions_Template.xlsx
+++ b/templates/CBX250_Model_Assumptions_Template.xlsx
@@ -182,12 +182,12 @@
       </c>
       <c r="B3" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Current scope covers Phase 1, Phase 2, and the active deterministic Phase 3 trade layer assumptions.</t>
+          <t xml:space="preserve">Current scope covers Phase 1, Phase 2, and the active deterministic Phase 3, Phase 4, and Phase 5 assumptions.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Production scheduling, inventory, financials, Monte Carlo, and UI remain later-phase work. Trade_Inventory_FutureHooks now wires the active deterministic Phase 3 trade config, but broader future-phase inventory behavior remains deferred.</t>
+          <t xml:space="preserve">Financials, Monte Carlo, and UI remain later-phase work. Trade_Inventory_FutureHooks now wires the active deterministic Phase 3 trade config plus the active deterministic Phase 4 scheduling and Phase 5 inventory configs.</t>
         </is>
       </c>
     </row>
@@ -250,12 +250,12 @@
       </c>
       <c r="B7" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">The importer generates machine-readable CSV artifacts plus generated_phase2_parameters.toml / generated_phase2_scenario.toml and generated_phase3_parameters.toml / generated_phase3_scenario.toml.</t>
+          <t xml:space="preserve">The importer generates machine-readable CSV artifacts plus generated_phase2_parameters.toml / generated_phase2_scenario.toml, generated_phase3_parameters.toml / generated_phase3_scenario.toml, generated_phase4_parameters.toml / generated_phase4_scenario.toml, and generated_phase5_parameters.toml / generated_phase5_scenario.toml.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Current wiring consumes: Scenario_Controls.demand_basis plus Treatment_Duration_Assumptions for Phase 1 starts-based mode; dose_basis_default, module-specific dosing values, module FG mg per unit, module FG vialing rule, global yields, DS quantity per DP unit default, DS overage default, SS ratio, and co_pack_mode for Phase 2; and active deterministic trade parameters from Trade_Inventory_FutureHooks for Phase 3.</t>
+          <t xml:space="preserve">Current wiring consumes: Scenario_Controls.demand_basis plus Treatment_Duration_Assumptions for Phase 1 starts-based mode; dose_basis_default, module-specific dosing values, module FG mg per unit, module FG vialing rule, global yields, DS quantity per DP unit default, DS overage default, SS ratio, and co_pack_mode for Phase 2; active deterministic trade parameters from Trade_Inventory_FutureHooks for Phase 3; and active deterministic Phase 4 scheduling plus Phase 5 inventory controls from Trade_Inventory_FutureHooks together with the scenario-default Product_Parameters, Yield_Assumptions, and SS_Assumptions rows.</t>
         </is>
       </c>
     </row>
@@ -272,7 +272,7 @@
       </c>
       <c r="C8" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">CML_Prevalent_Assumptions remains a dedicated artifact sheet. Populate approved pool, timing, and exhaustion metadata here without treating CML like AML/MDS segment mix logic. Trade_Inventory_FutureHooks still carries a historical name, but it now also feeds the active deterministic Phase 3 trade config.</t>
+          <t xml:space="preserve">CML_Prevalent_Assumptions remains a dedicated artifact sheet. Populate approved pool, timing, and exhaustion metadata here without treating CML like AML/MDS segment mix logic. Trade_Inventory_FutureHooks still carries a historical name, but it now also feeds the active deterministic Phase 3 trade config plus the active Phase 4 scheduling and Phase 5 inventory config bridges.</t>
         </is>
       </c>
     </row>
@@ -289,7 +289,7 @@
       </c>
       <c r="C9" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">This keeps the current architecture intact while removing the need to edit TOML by hand for the active deterministic assumptions. The workflow also consumes the generated treatment duration artifact when demand_basis = patient_starts and can optionally run through Phase 3.</t>
+          <t xml:space="preserve">This keeps the current architecture intact while removing the need to edit TOML by hand for the active deterministic assumptions. The workflow also consumes the generated treatment duration artifact when demand_basis = patient_starts and can optionally run through Phase 5.</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:BV21"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1165,8 +1165,58 @@
     <col min="19" max="19" width="20" customWidth="1"/>
     <col min="20" max="20" width="20" customWidth="1"/>
     <col min="21" max="21" width="18" customWidth="1"/>
-    <col min="22" max="22" width="12" customWidth="1"/>
-    <col min="23" max="23" width="72" customWidth="1"/>
+    <col min="22" max="22" width="18" customWidth="1"/>
+    <col min="23" max="23" width="18" customWidth="1"/>
+    <col min="24" max="24" width="18" customWidth="1"/>
+    <col min="25" max="25" width="18" customWidth="1"/>
+    <col min="26" max="26" width="18" customWidth="1"/>
+    <col min="27" max="27" width="18" customWidth="1"/>
+    <col min="28" max="28" width="18" customWidth="1"/>
+    <col min="29" max="29" width="18" customWidth="1"/>
+    <col min="30" max="30" width="18" customWidth="1"/>
+    <col min="31" max="31" width="18" customWidth="1"/>
+    <col min="32" max="32" width="18" customWidth="1"/>
+    <col min="33" max="33" width="20" customWidth="1"/>
+    <col min="34" max="34" width="18" customWidth="1"/>
+    <col min="35" max="35" width="18" customWidth="1"/>
+    <col min="36" max="36" width="18" customWidth="1"/>
+    <col min="37" max="37" width="18" customWidth="1"/>
+    <col min="38" max="38" width="20" customWidth="1"/>
+    <col min="39" max="39" width="20" customWidth="1"/>
+    <col min="40" max="40" width="18" customWidth="1"/>
+    <col min="41" max="41" width="18" customWidth="1"/>
+    <col min="42" max="42" width="18" customWidth="1"/>
+    <col min="43" max="43" width="22" customWidth="1"/>
+    <col min="44" max="44" width="18" customWidth="1"/>
+    <col min="45" max="45" width="18" customWidth="1"/>
+    <col min="46" max="46" width="18" customWidth="1"/>
+    <col min="47" max="47" width="18" customWidth="1"/>
+    <col min="48" max="48" width="18" customWidth="1"/>
+    <col min="49" max="49" width="18" customWidth="1"/>
+    <col min="50" max="50" width="18" customWidth="1"/>
+    <col min="51" max="51" width="18" customWidth="1"/>
+    <col min="52" max="52" width="18" customWidth="1"/>
+    <col min="53" max="53" width="18" customWidth="1"/>
+    <col min="54" max="54" width="18" customWidth="1"/>
+    <col min="55" max="55" width="18" customWidth="1"/>
+    <col min="56" max="56" width="18" customWidth="1"/>
+    <col min="57" max="57" width="18" customWidth="1"/>
+    <col min="58" max="58" width="18" customWidth="1"/>
+    <col min="59" max="59" width="18" customWidth="1"/>
+    <col min="60" max="60" width="18" customWidth="1"/>
+    <col min="61" max="61" width="18" customWidth="1"/>
+    <col min="62" max="62" width="18" customWidth="1"/>
+    <col min="63" max="63" width="18" customWidth="1"/>
+    <col min="64" max="64" width="18" customWidth="1"/>
+    <col min="65" max="65" width="18" customWidth="1"/>
+    <col min="66" max="66" width="18" customWidth="1"/>
+    <col min="67" max="67" width="18" customWidth="1"/>
+    <col min="68" max="68" width="18" customWidth="1"/>
+    <col min="69" max="69" width="18" customWidth="1"/>
+    <col min="70" max="70" width="18" customWidth="1"/>
+    <col min="71" max="71" width="18" customWidth="1"/>
+    <col min="72" max="72" width="12" customWidth="1"/>
+    <col min="73" max="73" width="72" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1277,10 +1327,265 @@
       </c>
       <c r="V1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">bullwhip_amplification_threshold</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">bullwhip_review_window_months</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">excess_build_threshold_ratio</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">supply_gap_tolerance_units</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">capacity_clip_tolerance_units</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">cml_prevalent_forward_window_months</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">projected_cml_prevalent_bolus_exhaustion_month_index</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">fg_lead_time_from_dp_release_weeks</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">fg_packaging_cycle_weeks</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">fg_release_qa_weeks</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">fg_total_order_to_release_weeks</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">fg_packaging_campaign_size_units</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_lead_time_from_ds_release_weeks</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_manufacturing_cycle_weeks</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_release_testing_weeks</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_total_order_to_release_weeks</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_min_batch_size_units</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_max_batch_size_units</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_min_campaign_batches</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_annual_capacity_batches</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_lead_time_to_batch_start_planning_horizon_weeks</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_manufacturing_cycle_weeks</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_release_testing_weeks</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_total_order_to_release_weeks</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_min_batch_size_kg</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_max_batch_size_kg</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_min_campaign_batches</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_annual_capacity_batches</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ss_order_to_release_lead_time_weeks</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ss_batch_size_units</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ss_min_campaign_batches</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ss_annual_capacity_batches</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ss_release_must_coincide_with_or_precede_fg</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">starting_inventory_ds_mg</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">starting_inventory_dp_units</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">starting_inventory_fg_units</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">starting_inventory_ss_units</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">starting_inventory_sublayer1_fg_units</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">starting_inventory_sublayer2_fg_units</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">shelf_life_ds_months</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">shelf_life_dp_months</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">shelf_life_fg_months</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">shelf_life_ss_months</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">excess_inventory_threshold_months_of_cover</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">stockout_tolerance_units</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">fefo_enabled</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ss_fg_match_required</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">allow_prelaunch_inventory_build</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">phase5_enforce_unique_output_keys</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">phase5_reconcile_phase4_receipts</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">phase5_reconciliation_tolerance_units</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">active_flag</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr" s="1">
+      <c r="BV1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">notes</t>
         </is>
@@ -1350,14 +1655,179 @@
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
-      <c r="V2" t="inlineStr" s="2">
+      <c r="V2" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="W2" s="2">
+        <v>2</v>
+      </c>
+      <c r="X2" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="Y2" s="2">
+        <v>1e-06</v>
+      </c>
+      <c r="Z2" s="2">
+        <v>1e-06</v>
+      </c>
+      <c r="AA2" s="2">
+        <v>6</v>
+      </c>
+      <c r="AB2" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="2">
+        <v>4</v>
+      </c>
+      <c r="AD2" s="2">
+        <v>2</v>
+      </c>
+      <c r="AE2" s="2">
+        <v>2</v>
+      </c>
+      <c r="AF2" s="2">
+        <v>8</v>
+      </c>
+      <c r="AG2" s="2">
+        <v>50000</v>
+      </c>
+      <c r="AH2" s="2">
+        <v>4</v>
+      </c>
+      <c r="AI2" s="2">
+        <v>2</v>
+      </c>
+      <c r="AJ2" s="2">
+        <v>12</v>
+      </c>
+      <c r="AK2" s="2">
+        <v>18</v>
+      </c>
+      <c r="AL2" s="2">
+        <v>100000</v>
+      </c>
+      <c r="AM2" s="2">
+        <v>500000</v>
+      </c>
+      <c r="AN2" s="2">
+        <v>3</v>
+      </c>
+      <c r="AO2" s="2">
+        <v>10</v>
+      </c>
+      <c r="AP2" s="2">
+        <v>24</v>
+      </c>
+      <c r="AQ2" s="2">
+        <v>8</v>
+      </c>
+      <c r="AR2" s="2">
+        <v>12</v>
+      </c>
+      <c r="AS2" s="2">
+        <v>44</v>
+      </c>
+      <c r="AT2" s="2">
+        <v>2</v>
+      </c>
+      <c r="AU2" s="2">
+        <v>4</v>
+      </c>
+      <c r="AV2" s="2">
+        <v>3</v>
+      </c>
+      <c r="AW2" s="2">
+        <v>5</v>
+      </c>
+      <c r="AX2" s="2">
+        <v>24</v>
+      </c>
+      <c r="AY2" s="2">
+        <v>100000</v>
+      </c>
+      <c r="AZ2" s="2">
+        <v>3</v>
+      </c>
+      <c r="BA2" s="2">
+        <v>10</v>
+      </c>
+      <c r="BB2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="BC2" s="2">
+        <v>0</v>
+      </c>
+      <c r="BD2" s="2">
+        <v>0</v>
+      </c>
+      <c r="BE2" s="2">
+        <v>0</v>
+      </c>
+      <c r="BF2" s="2">
+        <v>0</v>
+      </c>
+      <c r="BG2" s="2">
+        <v>0</v>
+      </c>
+      <c r="BH2" s="2">
+        <v>0</v>
+      </c>
+      <c r="BI2" s="2">
+        <v>24</v>
+      </c>
+      <c r="BJ2" s="2">
+        <v>24</v>
+      </c>
+      <c r="BK2" s="2">
+        <v>24</v>
+      </c>
+      <c r="BL2" s="2">
+        <v>24</v>
+      </c>
+      <c r="BM2" s="2">
+        <v>6</v>
+      </c>
+      <c r="BN2" s="2">
+        <v>1e-06</v>
+      </c>
+      <c r="BO2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="BQ2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="BR2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="BT2" s="2">
+        <v>1e-06</v>
+      </c>
+      <c r="BU2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">Approved deterministic Phase 3 scenario defaults. Edit here instead of phase3_trade_layer.toml.</t>
+      <c r="BV2" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Active deterministic defaults for Phase 3, Phase 4, and Phase 5. Edit here instead of hand-editing phase3_trade_layer.toml, phase4_production_schedule.toml, or phase5_inventory_layer.toml.</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1873,63 @@
         <v>25</v>
       </c>
       <c r="U3" s="2"/>
-      <c r="V3" t="inlineStr" s="2">
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="2"/>
+      <c r="AK3" s="2"/>
+      <c r="AL3" s="2"/>
+      <c r="AM3" s="2"/>
+      <c r="AN3" s="2"/>
+      <c r="AO3" s="2"/>
+      <c r="AP3" s="2"/>
+      <c r="AQ3" s="2"/>
+      <c r="AR3" s="2"/>
+      <c r="AS3" s="2"/>
+      <c r="AT3" s="2"/>
+      <c r="AU3" s="2"/>
+      <c r="AV3" s="2"/>
+      <c r="AW3" s="2"/>
+      <c r="AX3" s="2"/>
+      <c r="AY3" s="2"/>
+      <c r="AZ3" s="2"/>
+      <c r="BA3" s="2"/>
+      <c r="BB3" s="2"/>
+      <c r="BC3" s="2"/>
+      <c r="BD3" s="2"/>
+      <c r="BE3" s="2"/>
+      <c r="BF3" s="2"/>
+      <c r="BG3" s="2"/>
+      <c r="BH3" s="2"/>
+      <c r="BI3" s="2"/>
+      <c r="BJ3" s="2"/>
+      <c r="BK3" s="2"/>
+      <c r="BL3" s="2"/>
+      <c r="BM3" s="2"/>
+      <c r="BN3" s="2"/>
+      <c r="BO3" s="2"/>
+      <c r="BP3" s="2"/>
+      <c r="BQ3" s="2"/>
+      <c r="BR3" s="2"/>
+      <c r="BS3" s="2"/>
+      <c r="BT3" s="2"/>
+      <c r="BU3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr" s="9">
+      <c r="BV3" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample US site activation defaults for the deterministic Phase 3 trade layer.</t>
         </is>
@@ -1456,12 +1977,63 @@
         <v>18</v>
       </c>
       <c r="U4" s="2"/>
-      <c r="V4" t="inlineStr" s="2">
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="2"/>
+      <c r="AJ4" s="2"/>
+      <c r="AK4" s="2"/>
+      <c r="AL4" s="2"/>
+      <c r="AM4" s="2"/>
+      <c r="AN4" s="2"/>
+      <c r="AO4" s="2"/>
+      <c r="AP4" s="2"/>
+      <c r="AQ4" s="2"/>
+      <c r="AR4" s="2"/>
+      <c r="AS4" s="2"/>
+      <c r="AT4" s="2"/>
+      <c r="AU4" s="2"/>
+      <c r="AV4" s="2"/>
+      <c r="AW4" s="2"/>
+      <c r="AX4" s="2"/>
+      <c r="AY4" s="2"/>
+      <c r="AZ4" s="2"/>
+      <c r="BA4" s="2"/>
+      <c r="BB4" s="2"/>
+      <c r="BC4" s="2"/>
+      <c r="BD4" s="2"/>
+      <c r="BE4" s="2"/>
+      <c r="BF4" s="2"/>
+      <c r="BG4" s="2"/>
+      <c r="BH4" s="2"/>
+      <c r="BI4" s="2"/>
+      <c r="BJ4" s="2"/>
+      <c r="BK4" s="2"/>
+      <c r="BL4" s="2"/>
+      <c r="BM4" s="2"/>
+      <c r="BN4" s="2"/>
+      <c r="BO4" s="2"/>
+      <c r="BP4" s="2"/>
+      <c r="BQ4" s="2"/>
+      <c r="BR4" s="2"/>
+      <c r="BS4" s="2"/>
+      <c r="BT4" s="2"/>
+      <c r="BU4" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr" s="9">
+      <c r="BV4" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample EU site activation defaults for the deterministic Phase 3 trade layer.</t>
         </is>
@@ -1505,12 +2077,63 @@
       <c r="U5" s="2">
         <v>1</v>
       </c>
-      <c r="V5" t="inlineStr" s="2">
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
+      <c r="AI5" s="2"/>
+      <c r="AJ5" s="2"/>
+      <c r="AK5" s="2"/>
+      <c r="AL5" s="2"/>
+      <c r="AM5" s="2"/>
+      <c r="AN5" s="2"/>
+      <c r="AO5" s="2"/>
+      <c r="AP5" s="2"/>
+      <c r="AQ5" s="2"/>
+      <c r="AR5" s="2"/>
+      <c r="AS5" s="2"/>
+      <c r="AT5" s="2"/>
+      <c r="AU5" s="2"/>
+      <c r="AV5" s="2"/>
+      <c r="AW5" s="2"/>
+      <c r="AX5" s="2"/>
+      <c r="AY5" s="2"/>
+      <c r="AZ5" s="2"/>
+      <c r="BA5" s="2"/>
+      <c r="BB5" s="2"/>
+      <c r="BC5" s="2"/>
+      <c r="BD5" s="2"/>
+      <c r="BE5" s="2"/>
+      <c r="BF5" s="2"/>
+      <c r="BG5" s="2"/>
+      <c r="BH5" s="2"/>
+      <c r="BI5" s="2"/>
+      <c r="BJ5" s="2"/>
+      <c r="BK5" s="2"/>
+      <c r="BL5" s="2"/>
+      <c r="BM5" s="2"/>
+      <c r="BN5" s="2"/>
+      <c r="BO5" s="2"/>
+      <c r="BP5" s="2"/>
+      <c r="BQ5" s="2"/>
+      <c r="BR5" s="2"/>
+      <c r="BS5" s="2"/>
+      <c r="BT5" s="2"/>
+      <c r="BU5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr" s="9">
+      <c r="BV5" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
@@ -1554,12 +2177,63 @@
       <c r="U6" s="2">
         <v>1</v>
       </c>
-      <c r="V6" t="inlineStr" s="2">
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+      <c r="AJ6" s="2"/>
+      <c r="AK6" s="2"/>
+      <c r="AL6" s="2"/>
+      <c r="AM6" s="2"/>
+      <c r="AN6" s="2"/>
+      <c r="AO6" s="2"/>
+      <c r="AP6" s="2"/>
+      <c r="AQ6" s="2"/>
+      <c r="AR6" s="2"/>
+      <c r="AS6" s="2"/>
+      <c r="AT6" s="2"/>
+      <c r="AU6" s="2"/>
+      <c r="AV6" s="2"/>
+      <c r="AW6" s="2"/>
+      <c r="AX6" s="2"/>
+      <c r="AY6" s="2"/>
+      <c r="AZ6" s="2"/>
+      <c r="BA6" s="2"/>
+      <c r="BB6" s="2"/>
+      <c r="BC6" s="2"/>
+      <c r="BD6" s="2"/>
+      <c r="BE6" s="2"/>
+      <c r="BF6" s="2"/>
+      <c r="BG6" s="2"/>
+      <c r="BH6" s="2"/>
+      <c r="BI6" s="2"/>
+      <c r="BJ6" s="2"/>
+      <c r="BK6" s="2"/>
+      <c r="BL6" s="2"/>
+      <c r="BM6" s="2"/>
+      <c r="BN6" s="2"/>
+      <c r="BO6" s="2"/>
+      <c r="BP6" s="2"/>
+      <c r="BQ6" s="2"/>
+      <c r="BR6" s="2"/>
+      <c r="BS6" s="2"/>
+      <c r="BT6" s="2"/>
+      <c r="BU6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr" s="9">
+      <c r="BV6" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
@@ -1603,12 +2277,63 @@
       <c r="U7" s="2">
         <v>1</v>
       </c>
-      <c r="V7" t="inlineStr" s="2">
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+      <c r="AJ7" s="2"/>
+      <c r="AK7" s="2"/>
+      <c r="AL7" s="2"/>
+      <c r="AM7" s="2"/>
+      <c r="AN7" s="2"/>
+      <c r="AO7" s="2"/>
+      <c r="AP7" s="2"/>
+      <c r="AQ7" s="2"/>
+      <c r="AR7" s="2"/>
+      <c r="AS7" s="2"/>
+      <c r="AT7" s="2"/>
+      <c r="AU7" s="2"/>
+      <c r="AV7" s="2"/>
+      <c r="AW7" s="2"/>
+      <c r="AX7" s="2"/>
+      <c r="AY7" s="2"/>
+      <c r="AZ7" s="2"/>
+      <c r="BA7" s="2"/>
+      <c r="BB7" s="2"/>
+      <c r="BC7" s="2"/>
+      <c r="BD7" s="2"/>
+      <c r="BE7" s="2"/>
+      <c r="BF7" s="2"/>
+      <c r="BG7" s="2"/>
+      <c r="BH7" s="2"/>
+      <c r="BI7" s="2"/>
+      <c r="BJ7" s="2"/>
+      <c r="BK7" s="2"/>
+      <c r="BL7" s="2"/>
+      <c r="BM7" s="2"/>
+      <c r="BN7" s="2"/>
+      <c r="BO7" s="2"/>
+      <c r="BP7" s="2"/>
+      <c r="BQ7" s="2"/>
+      <c r="BR7" s="2"/>
+      <c r="BS7" s="2"/>
+      <c r="BT7" s="2"/>
+      <c r="BU7" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr" s="9">
+      <c r="BV7" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
@@ -1652,12 +2377,63 @@
       <c r="U8" s="2">
         <v>1</v>
       </c>
-      <c r="V8" t="inlineStr" s="2">
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+      <c r="X8" s="2"/>
+      <c r="Y8" s="2"/>
+      <c r="Z8" s="2"/>
+      <c r="AA8" s="2"/>
+      <c r="AB8" s="2"/>
+      <c r="AC8" s="2"/>
+      <c r="AD8" s="2"/>
+      <c r="AE8" s="2"/>
+      <c r="AF8" s="2"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="2"/>
+      <c r="AI8" s="2"/>
+      <c r="AJ8" s="2"/>
+      <c r="AK8" s="2"/>
+      <c r="AL8" s="2"/>
+      <c r="AM8" s="2"/>
+      <c r="AN8" s="2"/>
+      <c r="AO8" s="2"/>
+      <c r="AP8" s="2"/>
+      <c r="AQ8" s="2"/>
+      <c r="AR8" s="2"/>
+      <c r="AS8" s="2"/>
+      <c r="AT8" s="2"/>
+      <c r="AU8" s="2"/>
+      <c r="AV8" s="2"/>
+      <c r="AW8" s="2"/>
+      <c r="AX8" s="2"/>
+      <c r="AY8" s="2"/>
+      <c r="AZ8" s="2"/>
+      <c r="BA8" s="2"/>
+      <c r="BB8" s="2"/>
+      <c r="BC8" s="2"/>
+      <c r="BD8" s="2"/>
+      <c r="BE8" s="2"/>
+      <c r="BF8" s="2"/>
+      <c r="BG8" s="2"/>
+      <c r="BH8" s="2"/>
+      <c r="BI8" s="2"/>
+      <c r="BJ8" s="2"/>
+      <c r="BK8" s="2"/>
+      <c r="BL8" s="2"/>
+      <c r="BM8" s="2"/>
+      <c r="BN8" s="2"/>
+      <c r="BO8" s="2"/>
+      <c r="BP8" s="2"/>
+      <c r="BQ8" s="2"/>
+      <c r="BR8" s="2"/>
+      <c r="BS8" s="2"/>
+      <c r="BT8" s="2"/>
+      <c r="BU8" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr" s="9">
+      <c r="BV8" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
@@ -1701,12 +2477,63 @@
       <c r="U9" s="2">
         <v>1</v>
       </c>
-      <c r="V9" t="inlineStr" s="2">
+      <c r="V9" s="2"/>
+      <c r="W9" s="2"/>
+      <c r="X9" s="2"/>
+      <c r="Y9" s="2"/>
+      <c r="Z9" s="2"/>
+      <c r="AA9" s="2"/>
+      <c r="AB9" s="2"/>
+      <c r="AC9" s="2"/>
+      <c r="AD9" s="2"/>
+      <c r="AE9" s="2"/>
+      <c r="AF9" s="2"/>
+      <c r="AG9" s="2"/>
+      <c r="AH9" s="2"/>
+      <c r="AI9" s="2"/>
+      <c r="AJ9" s="2"/>
+      <c r="AK9" s="2"/>
+      <c r="AL9" s="2"/>
+      <c r="AM9" s="2"/>
+      <c r="AN9" s="2"/>
+      <c r="AO9" s="2"/>
+      <c r="AP9" s="2"/>
+      <c r="AQ9" s="2"/>
+      <c r="AR9" s="2"/>
+      <c r="AS9" s="2"/>
+      <c r="AT9" s="2"/>
+      <c r="AU9" s="2"/>
+      <c r="AV9" s="2"/>
+      <c r="AW9" s="2"/>
+      <c r="AX9" s="2"/>
+      <c r="AY9" s="2"/>
+      <c r="AZ9" s="2"/>
+      <c r="BA9" s="2"/>
+      <c r="BB9" s="2"/>
+      <c r="BC9" s="2"/>
+      <c r="BD9" s="2"/>
+      <c r="BE9" s="2"/>
+      <c r="BF9" s="2"/>
+      <c r="BG9" s="2"/>
+      <c r="BH9" s="2"/>
+      <c r="BI9" s="2"/>
+      <c r="BJ9" s="2"/>
+      <c r="BK9" s="2"/>
+      <c r="BL9" s="2"/>
+      <c r="BM9" s="2"/>
+      <c r="BN9" s="2"/>
+      <c r="BO9" s="2"/>
+      <c r="BP9" s="2"/>
+      <c r="BQ9" s="2"/>
+      <c r="BR9" s="2"/>
+      <c r="BS9" s="2"/>
+      <c r="BT9" s="2"/>
+      <c r="BU9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr" s="9">
+      <c r="BV9" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
@@ -1750,12 +2577,63 @@
       <c r="U10" s="2">
         <v>1</v>
       </c>
-      <c r="V10" t="inlineStr" s="2">
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
+      <c r="X10" s="2"/>
+      <c r="Y10" s="2"/>
+      <c r="Z10" s="2"/>
+      <c r="AA10" s="2"/>
+      <c r="AB10" s="2"/>
+      <c r="AC10" s="2"/>
+      <c r="AD10" s="2"/>
+      <c r="AE10" s="2"/>
+      <c r="AF10" s="2"/>
+      <c r="AG10" s="2"/>
+      <c r="AH10" s="2"/>
+      <c r="AI10" s="2"/>
+      <c r="AJ10" s="2"/>
+      <c r="AK10" s="2"/>
+      <c r="AL10" s="2"/>
+      <c r="AM10" s="2"/>
+      <c r="AN10" s="2"/>
+      <c r="AO10" s="2"/>
+      <c r="AP10" s="2"/>
+      <c r="AQ10" s="2"/>
+      <c r="AR10" s="2"/>
+      <c r="AS10" s="2"/>
+      <c r="AT10" s="2"/>
+      <c r="AU10" s="2"/>
+      <c r="AV10" s="2"/>
+      <c r="AW10" s="2"/>
+      <c r="AX10" s="2"/>
+      <c r="AY10" s="2"/>
+      <c r="AZ10" s="2"/>
+      <c r="BA10" s="2"/>
+      <c r="BB10" s="2"/>
+      <c r="BC10" s="2"/>
+      <c r="BD10" s="2"/>
+      <c r="BE10" s="2"/>
+      <c r="BF10" s="2"/>
+      <c r="BG10" s="2"/>
+      <c r="BH10" s="2"/>
+      <c r="BI10" s="2"/>
+      <c r="BJ10" s="2"/>
+      <c r="BK10" s="2"/>
+      <c r="BL10" s="2"/>
+      <c r="BM10" s="2"/>
+      <c r="BN10" s="2"/>
+      <c r="BO10" s="2"/>
+      <c r="BP10" s="2"/>
+      <c r="BQ10" s="2"/>
+      <c r="BR10" s="2"/>
+      <c r="BS10" s="2"/>
+      <c r="BT10" s="2"/>
+      <c r="BU10" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr" s="9">
+      <c r="BV10" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
@@ -1799,12 +2677,63 @@
       <c r="U11" s="2">
         <v>1</v>
       </c>
-      <c r="V11" t="inlineStr" s="2">
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
+      <c r="Y11" s="2"/>
+      <c r="Z11" s="2"/>
+      <c r="AA11" s="2"/>
+      <c r="AB11" s="2"/>
+      <c r="AC11" s="2"/>
+      <c r="AD11" s="2"/>
+      <c r="AE11" s="2"/>
+      <c r="AF11" s="2"/>
+      <c r="AG11" s="2"/>
+      <c r="AH11" s="2"/>
+      <c r="AI11" s="2"/>
+      <c r="AJ11" s="2"/>
+      <c r="AK11" s="2"/>
+      <c r="AL11" s="2"/>
+      <c r="AM11" s="2"/>
+      <c r="AN11" s="2"/>
+      <c r="AO11" s="2"/>
+      <c r="AP11" s="2"/>
+      <c r="AQ11" s="2"/>
+      <c r="AR11" s="2"/>
+      <c r="AS11" s="2"/>
+      <c r="AT11" s="2"/>
+      <c r="AU11" s="2"/>
+      <c r="AV11" s="2"/>
+      <c r="AW11" s="2"/>
+      <c r="AX11" s="2"/>
+      <c r="AY11" s="2"/>
+      <c r="AZ11" s="2"/>
+      <c r="BA11" s="2"/>
+      <c r="BB11" s="2"/>
+      <c r="BC11" s="2"/>
+      <c r="BD11" s="2"/>
+      <c r="BE11" s="2"/>
+      <c r="BF11" s="2"/>
+      <c r="BG11" s="2"/>
+      <c r="BH11" s="2"/>
+      <c r="BI11" s="2"/>
+      <c r="BJ11" s="2"/>
+      <c r="BK11" s="2"/>
+      <c r="BL11" s="2"/>
+      <c r="BM11" s="2"/>
+      <c r="BN11" s="2"/>
+      <c r="BO11" s="2"/>
+      <c r="BP11" s="2"/>
+      <c r="BQ11" s="2"/>
+      <c r="BR11" s="2"/>
+      <c r="BS11" s="2"/>
+      <c r="BT11" s="2"/>
+      <c r="BU11" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr" s="9">
+      <c r="BV11" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
@@ -1848,12 +2777,63 @@
       <c r="U12" s="2">
         <v>1</v>
       </c>
-      <c r="V12" t="inlineStr" s="2">
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
+      <c r="X12" s="2"/>
+      <c r="Y12" s="2"/>
+      <c r="Z12" s="2"/>
+      <c r="AA12" s="2"/>
+      <c r="AB12" s="2"/>
+      <c r="AC12" s="2"/>
+      <c r="AD12" s="2"/>
+      <c r="AE12" s="2"/>
+      <c r="AF12" s="2"/>
+      <c r="AG12" s="2"/>
+      <c r="AH12" s="2"/>
+      <c r="AI12" s="2"/>
+      <c r="AJ12" s="2"/>
+      <c r="AK12" s="2"/>
+      <c r="AL12" s="2"/>
+      <c r="AM12" s="2"/>
+      <c r="AN12" s="2"/>
+      <c r="AO12" s="2"/>
+      <c r="AP12" s="2"/>
+      <c r="AQ12" s="2"/>
+      <c r="AR12" s="2"/>
+      <c r="AS12" s="2"/>
+      <c r="AT12" s="2"/>
+      <c r="AU12" s="2"/>
+      <c r="AV12" s="2"/>
+      <c r="AW12" s="2"/>
+      <c r="AX12" s="2"/>
+      <c r="AY12" s="2"/>
+      <c r="AZ12" s="2"/>
+      <c r="BA12" s="2"/>
+      <c r="BB12" s="2"/>
+      <c r="BC12" s="2"/>
+      <c r="BD12" s="2"/>
+      <c r="BE12" s="2"/>
+      <c r="BF12" s="2"/>
+      <c r="BG12" s="2"/>
+      <c r="BH12" s="2"/>
+      <c r="BI12" s="2"/>
+      <c r="BJ12" s="2"/>
+      <c r="BK12" s="2"/>
+      <c r="BL12" s="2"/>
+      <c r="BM12" s="2"/>
+      <c r="BN12" s="2"/>
+      <c r="BO12" s="2"/>
+      <c r="BP12" s="2"/>
+      <c r="BQ12" s="2"/>
+      <c r="BR12" s="2"/>
+      <c r="BS12" s="2"/>
+      <c r="BT12" s="2"/>
+      <c r="BU12" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr" s="9">
+      <c r="BV12" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
@@ -1882,7 +2862,58 @@
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
-      <c r="W13" s="9"/>
+      <c r="W13" s="2"/>
+      <c r="X13" s="2"/>
+      <c r="Y13" s="2"/>
+      <c r="Z13" s="2"/>
+      <c r="AA13" s="2"/>
+      <c r="AB13" s="2"/>
+      <c r="AC13" s="2"/>
+      <c r="AD13" s="2"/>
+      <c r="AE13" s="2"/>
+      <c r="AF13" s="2"/>
+      <c r="AG13" s="2"/>
+      <c r="AH13" s="2"/>
+      <c r="AI13" s="2"/>
+      <c r="AJ13" s="2"/>
+      <c r="AK13" s="2"/>
+      <c r="AL13" s="2"/>
+      <c r="AM13" s="2"/>
+      <c r="AN13" s="2"/>
+      <c r="AO13" s="2"/>
+      <c r="AP13" s="2"/>
+      <c r="AQ13" s="2"/>
+      <c r="AR13" s="2"/>
+      <c r="AS13" s="2"/>
+      <c r="AT13" s="2"/>
+      <c r="AU13" s="2"/>
+      <c r="AV13" s="2"/>
+      <c r="AW13" s="2"/>
+      <c r="AX13" s="2"/>
+      <c r="AY13" s="2"/>
+      <c r="AZ13" s="2"/>
+      <c r="BA13" s="2"/>
+      <c r="BB13" s="2"/>
+      <c r="BC13" s="2"/>
+      <c r="BD13" s="2"/>
+      <c r="BE13" s="2"/>
+      <c r="BF13" s="2"/>
+      <c r="BG13" s="2"/>
+      <c r="BH13" s="2"/>
+      <c r="BI13" s="2"/>
+      <c r="BJ13" s="2"/>
+      <c r="BK13" s="2"/>
+      <c r="BL13" s="2"/>
+      <c r="BM13" s="2"/>
+      <c r="BN13" s="2"/>
+      <c r="BO13" s="2"/>
+      <c r="BP13" s="2"/>
+      <c r="BQ13" s="2"/>
+      <c r="BR13" s="2"/>
+      <c r="BS13" s="2"/>
+      <c r="BT13" s="2"/>
+      <c r="BU13" s="2"/>
+      <c r="BV13" s="9"/>
     </row>
     <row r="14">
       <c r="A14" s="3"/>
@@ -1907,7 +2938,58 @@
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
-      <c r="W14" s="9"/>
+      <c r="W14" s="2"/>
+      <c r="X14" s="2"/>
+      <c r="Y14" s="2"/>
+      <c r="Z14" s="2"/>
+      <c r="AA14" s="2"/>
+      <c r="AB14" s="2"/>
+      <c r="AC14" s="2"/>
+      <c r="AD14" s="2"/>
+      <c r="AE14" s="2"/>
+      <c r="AF14" s="2"/>
+      <c r="AG14" s="2"/>
+      <c r="AH14" s="2"/>
+      <c r="AI14" s="2"/>
+      <c r="AJ14" s="2"/>
+      <c r="AK14" s="2"/>
+      <c r="AL14" s="2"/>
+      <c r="AM14" s="2"/>
+      <c r="AN14" s="2"/>
+      <c r="AO14" s="2"/>
+      <c r="AP14" s="2"/>
+      <c r="AQ14" s="2"/>
+      <c r="AR14" s="2"/>
+      <c r="AS14" s="2"/>
+      <c r="AT14" s="2"/>
+      <c r="AU14" s="2"/>
+      <c r="AV14" s="2"/>
+      <c r="AW14" s="2"/>
+      <c r="AX14" s="2"/>
+      <c r="AY14" s="2"/>
+      <c r="AZ14" s="2"/>
+      <c r="BA14" s="2"/>
+      <c r="BB14" s="2"/>
+      <c r="BC14" s="2"/>
+      <c r="BD14" s="2"/>
+      <c r="BE14" s="2"/>
+      <c r="BF14" s="2"/>
+      <c r="BG14" s="2"/>
+      <c r="BH14" s="2"/>
+      <c r="BI14" s="2"/>
+      <c r="BJ14" s="2"/>
+      <c r="BK14" s="2"/>
+      <c r="BL14" s="2"/>
+      <c r="BM14" s="2"/>
+      <c r="BN14" s="2"/>
+      <c r="BO14" s="2"/>
+      <c r="BP14" s="2"/>
+      <c r="BQ14" s="2"/>
+      <c r="BR14" s="2"/>
+      <c r="BS14" s="2"/>
+      <c r="BT14" s="2"/>
+      <c r="BU14" s="2"/>
+      <c r="BV14" s="9"/>
     </row>
     <row r="15">
       <c r="A15" s="3"/>
@@ -1932,7 +3014,58 @@
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
-      <c r="W15" s="9"/>
+      <c r="W15" s="2"/>
+      <c r="X15" s="2"/>
+      <c r="Y15" s="2"/>
+      <c r="Z15" s="2"/>
+      <c r="AA15" s="2"/>
+      <c r="AB15" s="2"/>
+      <c r="AC15" s="2"/>
+      <c r="AD15" s="2"/>
+      <c r="AE15" s="2"/>
+      <c r="AF15" s="2"/>
+      <c r="AG15" s="2"/>
+      <c r="AH15" s="2"/>
+      <c r="AI15" s="2"/>
+      <c r="AJ15" s="2"/>
+      <c r="AK15" s="2"/>
+      <c r="AL15" s="2"/>
+      <c r="AM15" s="2"/>
+      <c r="AN15" s="2"/>
+      <c r="AO15" s="2"/>
+      <c r="AP15" s="2"/>
+      <c r="AQ15" s="2"/>
+      <c r="AR15" s="2"/>
+      <c r="AS15" s="2"/>
+      <c r="AT15" s="2"/>
+      <c r="AU15" s="2"/>
+      <c r="AV15" s="2"/>
+      <c r="AW15" s="2"/>
+      <c r="AX15" s="2"/>
+      <c r="AY15" s="2"/>
+      <c r="AZ15" s="2"/>
+      <c r="BA15" s="2"/>
+      <c r="BB15" s="2"/>
+      <c r="BC15" s="2"/>
+      <c r="BD15" s="2"/>
+      <c r="BE15" s="2"/>
+      <c r="BF15" s="2"/>
+      <c r="BG15" s="2"/>
+      <c r="BH15" s="2"/>
+      <c r="BI15" s="2"/>
+      <c r="BJ15" s="2"/>
+      <c r="BK15" s="2"/>
+      <c r="BL15" s="2"/>
+      <c r="BM15" s="2"/>
+      <c r="BN15" s="2"/>
+      <c r="BO15" s="2"/>
+      <c r="BP15" s="2"/>
+      <c r="BQ15" s="2"/>
+      <c r="BR15" s="2"/>
+      <c r="BS15" s="2"/>
+      <c r="BT15" s="2"/>
+      <c r="BU15" s="2"/>
+      <c r="BV15" s="9"/>
     </row>
     <row r="16">
       <c r="A16" s="3"/>
@@ -1957,7 +3090,58 @@
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
-      <c r="W16" s="9"/>
+      <c r="W16" s="2"/>
+      <c r="X16" s="2"/>
+      <c r="Y16" s="2"/>
+      <c r="Z16" s="2"/>
+      <c r="AA16" s="2"/>
+      <c r="AB16" s="2"/>
+      <c r="AC16" s="2"/>
+      <c r="AD16" s="2"/>
+      <c r="AE16" s="2"/>
+      <c r="AF16" s="2"/>
+      <c r="AG16" s="2"/>
+      <c r="AH16" s="2"/>
+      <c r="AI16" s="2"/>
+      <c r="AJ16" s="2"/>
+      <c r="AK16" s="2"/>
+      <c r="AL16" s="2"/>
+      <c r="AM16" s="2"/>
+      <c r="AN16" s="2"/>
+      <c r="AO16" s="2"/>
+      <c r="AP16" s="2"/>
+      <c r="AQ16" s="2"/>
+      <c r="AR16" s="2"/>
+      <c r="AS16" s="2"/>
+      <c r="AT16" s="2"/>
+      <c r="AU16" s="2"/>
+      <c r="AV16" s="2"/>
+      <c r="AW16" s="2"/>
+      <c r="AX16" s="2"/>
+      <c r="AY16" s="2"/>
+      <c r="AZ16" s="2"/>
+      <c r="BA16" s="2"/>
+      <c r="BB16" s="2"/>
+      <c r="BC16" s="2"/>
+      <c r="BD16" s="2"/>
+      <c r="BE16" s="2"/>
+      <c r="BF16" s="2"/>
+      <c r="BG16" s="2"/>
+      <c r="BH16" s="2"/>
+      <c r="BI16" s="2"/>
+      <c r="BJ16" s="2"/>
+      <c r="BK16" s="2"/>
+      <c r="BL16" s="2"/>
+      <c r="BM16" s="2"/>
+      <c r="BN16" s="2"/>
+      <c r="BO16" s="2"/>
+      <c r="BP16" s="2"/>
+      <c r="BQ16" s="2"/>
+      <c r="BR16" s="2"/>
+      <c r="BS16" s="2"/>
+      <c r="BT16" s="2"/>
+      <c r="BU16" s="2"/>
+      <c r="BV16" s="9"/>
     </row>
     <row r="17">
       <c r="A17" s="3"/>
@@ -1982,7 +3166,58 @@
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
-      <c r="W17" s="9"/>
+      <c r="W17" s="2"/>
+      <c r="X17" s="2"/>
+      <c r="Y17" s="2"/>
+      <c r="Z17" s="2"/>
+      <c r="AA17" s="2"/>
+      <c r="AB17" s="2"/>
+      <c r="AC17" s="2"/>
+      <c r="AD17" s="2"/>
+      <c r="AE17" s="2"/>
+      <c r="AF17" s="2"/>
+      <c r="AG17" s="2"/>
+      <c r="AH17" s="2"/>
+      <c r="AI17" s="2"/>
+      <c r="AJ17" s="2"/>
+      <c r="AK17" s="2"/>
+      <c r="AL17" s="2"/>
+      <c r="AM17" s="2"/>
+      <c r="AN17" s="2"/>
+      <c r="AO17" s="2"/>
+      <c r="AP17" s="2"/>
+      <c r="AQ17" s="2"/>
+      <c r="AR17" s="2"/>
+      <c r="AS17" s="2"/>
+      <c r="AT17" s="2"/>
+      <c r="AU17" s="2"/>
+      <c r="AV17" s="2"/>
+      <c r="AW17" s="2"/>
+      <c r="AX17" s="2"/>
+      <c r="AY17" s="2"/>
+      <c r="AZ17" s="2"/>
+      <c r="BA17" s="2"/>
+      <c r="BB17" s="2"/>
+      <c r="BC17" s="2"/>
+      <c r="BD17" s="2"/>
+      <c r="BE17" s="2"/>
+      <c r="BF17" s="2"/>
+      <c r="BG17" s="2"/>
+      <c r="BH17" s="2"/>
+      <c r="BI17" s="2"/>
+      <c r="BJ17" s="2"/>
+      <c r="BK17" s="2"/>
+      <c r="BL17" s="2"/>
+      <c r="BM17" s="2"/>
+      <c r="BN17" s="2"/>
+      <c r="BO17" s="2"/>
+      <c r="BP17" s="2"/>
+      <c r="BQ17" s="2"/>
+      <c r="BR17" s="2"/>
+      <c r="BS17" s="2"/>
+      <c r="BT17" s="2"/>
+      <c r="BU17" s="2"/>
+      <c r="BV17" s="9"/>
     </row>
     <row r="18">
       <c r="A18" s="3"/>
@@ -2007,7 +3242,58 @@
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
-      <c r="W18" s="9"/>
+      <c r="W18" s="2"/>
+      <c r="X18" s="2"/>
+      <c r="Y18" s="2"/>
+      <c r="Z18" s="2"/>
+      <c r="AA18" s="2"/>
+      <c r="AB18" s="2"/>
+      <c r="AC18" s="2"/>
+      <c r="AD18" s="2"/>
+      <c r="AE18" s="2"/>
+      <c r="AF18" s="2"/>
+      <c r="AG18" s="2"/>
+      <c r="AH18" s="2"/>
+      <c r="AI18" s="2"/>
+      <c r="AJ18" s="2"/>
+      <c r="AK18" s="2"/>
+      <c r="AL18" s="2"/>
+      <c r="AM18" s="2"/>
+      <c r="AN18" s="2"/>
+      <c r="AO18" s="2"/>
+      <c r="AP18" s="2"/>
+      <c r="AQ18" s="2"/>
+      <c r="AR18" s="2"/>
+      <c r="AS18" s="2"/>
+      <c r="AT18" s="2"/>
+      <c r="AU18" s="2"/>
+      <c r="AV18" s="2"/>
+      <c r="AW18" s="2"/>
+      <c r="AX18" s="2"/>
+      <c r="AY18" s="2"/>
+      <c r="AZ18" s="2"/>
+      <c r="BA18" s="2"/>
+      <c r="BB18" s="2"/>
+      <c r="BC18" s="2"/>
+      <c r="BD18" s="2"/>
+      <c r="BE18" s="2"/>
+      <c r="BF18" s="2"/>
+      <c r="BG18" s="2"/>
+      <c r="BH18" s="2"/>
+      <c r="BI18" s="2"/>
+      <c r="BJ18" s="2"/>
+      <c r="BK18" s="2"/>
+      <c r="BL18" s="2"/>
+      <c r="BM18" s="2"/>
+      <c r="BN18" s="2"/>
+      <c r="BO18" s="2"/>
+      <c r="BP18" s="2"/>
+      <c r="BQ18" s="2"/>
+      <c r="BR18" s="2"/>
+      <c r="BS18" s="2"/>
+      <c r="BT18" s="2"/>
+      <c r="BU18" s="2"/>
+      <c r="BV18" s="9"/>
     </row>
     <row r="19">
       <c r="A19" s="3"/>
@@ -2032,7 +3318,58 @@
       <c r="T19" s="2"/>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
-      <c r="W19" s="9"/>
+      <c r="W19" s="2"/>
+      <c r="X19" s="2"/>
+      <c r="Y19" s="2"/>
+      <c r="Z19" s="2"/>
+      <c r="AA19" s="2"/>
+      <c r="AB19" s="2"/>
+      <c r="AC19" s="2"/>
+      <c r="AD19" s="2"/>
+      <c r="AE19" s="2"/>
+      <c r="AF19" s="2"/>
+      <c r="AG19" s="2"/>
+      <c r="AH19" s="2"/>
+      <c r="AI19" s="2"/>
+      <c r="AJ19" s="2"/>
+      <c r="AK19" s="2"/>
+      <c r="AL19" s="2"/>
+      <c r="AM19" s="2"/>
+      <c r="AN19" s="2"/>
+      <c r="AO19" s="2"/>
+      <c r="AP19" s="2"/>
+      <c r="AQ19" s="2"/>
+      <c r="AR19" s="2"/>
+      <c r="AS19" s="2"/>
+      <c r="AT19" s="2"/>
+      <c r="AU19" s="2"/>
+      <c r="AV19" s="2"/>
+      <c r="AW19" s="2"/>
+      <c r="AX19" s="2"/>
+      <c r="AY19" s="2"/>
+      <c r="AZ19" s="2"/>
+      <c r="BA19" s="2"/>
+      <c r="BB19" s="2"/>
+      <c r="BC19" s="2"/>
+      <c r="BD19" s="2"/>
+      <c r="BE19" s="2"/>
+      <c r="BF19" s="2"/>
+      <c r="BG19" s="2"/>
+      <c r="BH19" s="2"/>
+      <c r="BI19" s="2"/>
+      <c r="BJ19" s="2"/>
+      <c r="BK19" s="2"/>
+      <c r="BL19" s="2"/>
+      <c r="BM19" s="2"/>
+      <c r="BN19" s="2"/>
+      <c r="BO19" s="2"/>
+      <c r="BP19" s="2"/>
+      <c r="BQ19" s="2"/>
+      <c r="BR19" s="2"/>
+      <c r="BS19" s="2"/>
+      <c r="BT19" s="2"/>
+      <c r="BU19" s="2"/>
+      <c r="BV19" s="9"/>
     </row>
     <row r="20">
       <c r="A20" s="3"/>
@@ -2057,7 +3394,58 @@
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
-      <c r="W20" s="9"/>
+      <c r="W20" s="2"/>
+      <c r="X20" s="2"/>
+      <c r="Y20" s="2"/>
+      <c r="Z20" s="2"/>
+      <c r="AA20" s="2"/>
+      <c r="AB20" s="2"/>
+      <c r="AC20" s="2"/>
+      <c r="AD20" s="2"/>
+      <c r="AE20" s="2"/>
+      <c r="AF20" s="2"/>
+      <c r="AG20" s="2"/>
+      <c r="AH20" s="2"/>
+      <c r="AI20" s="2"/>
+      <c r="AJ20" s="2"/>
+      <c r="AK20" s="2"/>
+      <c r="AL20" s="2"/>
+      <c r="AM20" s="2"/>
+      <c r="AN20" s="2"/>
+      <c r="AO20" s="2"/>
+      <c r="AP20" s="2"/>
+      <c r="AQ20" s="2"/>
+      <c r="AR20" s="2"/>
+      <c r="AS20" s="2"/>
+      <c r="AT20" s="2"/>
+      <c r="AU20" s="2"/>
+      <c r="AV20" s="2"/>
+      <c r="AW20" s="2"/>
+      <c r="AX20" s="2"/>
+      <c r="AY20" s="2"/>
+      <c r="AZ20" s="2"/>
+      <c r="BA20" s="2"/>
+      <c r="BB20" s="2"/>
+      <c r="BC20" s="2"/>
+      <c r="BD20" s="2"/>
+      <c r="BE20" s="2"/>
+      <c r="BF20" s="2"/>
+      <c r="BG20" s="2"/>
+      <c r="BH20" s="2"/>
+      <c r="BI20" s="2"/>
+      <c r="BJ20" s="2"/>
+      <c r="BK20" s="2"/>
+      <c r="BL20" s="2"/>
+      <c r="BM20" s="2"/>
+      <c r="BN20" s="2"/>
+      <c r="BO20" s="2"/>
+      <c r="BP20" s="2"/>
+      <c r="BQ20" s="2"/>
+      <c r="BR20" s="2"/>
+      <c r="BS20" s="2"/>
+      <c r="BT20" s="2"/>
+      <c r="BU20" s="2"/>
+      <c r="BV20" s="9"/>
     </row>
     <row r="21">
       <c r="A21" s="3"/>
@@ -2082,11 +3470,62 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="9"/>
+      <c r="W21" s="2"/>
+      <c r="X21" s="2"/>
+      <c r="Y21" s="2"/>
+      <c r="Z21" s="2"/>
+      <c r="AA21" s="2"/>
+      <c r="AB21" s="2"/>
+      <c r="AC21" s="2"/>
+      <c r="AD21" s="2"/>
+      <c r="AE21" s="2"/>
+      <c r="AF21" s="2"/>
+      <c r="AG21" s="2"/>
+      <c r="AH21" s="2"/>
+      <c r="AI21" s="2"/>
+      <c r="AJ21" s="2"/>
+      <c r="AK21" s="2"/>
+      <c r="AL21" s="2"/>
+      <c r="AM21" s="2"/>
+      <c r="AN21" s="2"/>
+      <c r="AO21" s="2"/>
+      <c r="AP21" s="2"/>
+      <c r="AQ21" s="2"/>
+      <c r="AR21" s="2"/>
+      <c r="AS21" s="2"/>
+      <c r="AT21" s="2"/>
+      <c r="AU21" s="2"/>
+      <c r="AV21" s="2"/>
+      <c r="AW21" s="2"/>
+      <c r="AX21" s="2"/>
+      <c r="AY21" s="2"/>
+      <c r="AZ21" s="2"/>
+      <c r="BA21" s="2"/>
+      <c r="BB21" s="2"/>
+      <c r="BC21" s="2"/>
+      <c r="BD21" s="2"/>
+      <c r="BE21" s="2"/>
+      <c r="BF21" s="2"/>
+      <c r="BG21" s="2"/>
+      <c r="BH21" s="2"/>
+      <c r="BI21" s="2"/>
+      <c r="BJ21" s="2"/>
+      <c r="BK21" s="2"/>
+      <c r="BL21" s="2"/>
+      <c r="BM21" s="2"/>
+      <c r="BN21" s="2"/>
+      <c r="BO21" s="2"/>
+      <c r="BP21" s="2"/>
+      <c r="BQ21" s="2"/>
+      <c r="BR21" s="2"/>
+      <c r="BS21" s="2"/>
+      <c r="BT21" s="2"/>
+      <c r="BU21" s="2"/>
+      <c r="BV21" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W1"/>
-  <dataValidations count="4">
+  <autoFilter ref="A1:BV1"/>
+  <dataValidations count="6">
     <dataValidation type="list" sqref="B2:B21" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$O$2:$O$4</formula1>
     </dataValidation>
@@ -2096,7 +3535,13 @@
     <dataValidation type="list" sqref="L2:L21" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$F$2:$F$3</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="V2:V21" showErrorMessage="1" allowBlank="1">
+    <dataValidation type="list" sqref="BB2:BB21" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="BO2:BS21" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="BU2:BU21" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$J$2:$J$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Lock Phase 5 deterministic inventory, shared scheduling grain, and policy calibration
</commit_message>
<xml_diff>
--- a/templates/CBX250_Model_Assumptions_Template.xlsx
+++ b/templates/CBX250_Model_Assumptions_Template.xlsx
@@ -1775,19 +1775,19 @@
         <v>0</v>
       </c>
       <c r="BI2" s="2">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="BJ2" s="2">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="BK2" s="2">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="BL2" s="2">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="BM2" s="2">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="BN2" s="2">
         <v>1e-06</v>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="BV2" t="inlineStr" s="9">
         <is>
-          <t xml:space="preserve">Active deterministic defaults for Phase 3, Phase 4, and Phase 5. Edit here instead of hand-editing phase3_trade_layer.toml, phase4_production_schedule.toml, or phase5_inventory_layer.toml.</t>
+          <t xml:space="preserve">Active deterministic defaults for Phase 3, Phase 4, and Phase 5. Phase 5 shelf life and excess-cover values are revised placeholder baseline assumptions; edit here instead of hand-editing phase3_trade_layer.toml, phase4_production_schedule.toml, or phase5_inventory_layer.toml.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock Updated Phase 6 layer
</commit_message>
<xml_diff>
--- a/templates/CBX250_Model_Assumptions_Template.xlsx
+++ b/templates/CBX250_Model_Assumptions_Template.xlsx
@@ -187,7 +187,7 @@
       </c>
       <c r="C3" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Financials, Monte Carlo, and UI remain later-phase work. Trade_Inventory_FutureHooks now wires the active deterministic Phase 3 trade config plus the active deterministic Phase 4 scheduling and Phase 5 inventory configs.</t>
+          <t xml:space="preserve">Revenue, Monte Carlo, and UI remain later-phase work. Trade_Inventory_FutureHooks now wires the active deterministic Phase 3 trade config plus the active deterministic Phase 4 scheduling, Phase 5 inventory, and Phase 6 financial configs.</t>
         </is>
       </c>
     </row>
@@ -250,12 +250,12 @@
       </c>
       <c r="B7" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">The importer generates machine-readable CSV artifacts plus generated_phase2_parameters.toml / generated_phase2_scenario.toml, generated_phase3_parameters.toml / generated_phase3_scenario.toml, generated_phase4_parameters.toml / generated_phase4_scenario.toml, and generated_phase5_parameters.toml / generated_phase5_scenario.toml.</t>
+          <t xml:space="preserve">The importer generates machine-readable CSV artifacts plus generated_phase2_parameters.toml / generated_phase2_scenario.toml, generated_phase3_parameters.toml / generated_phase3_scenario.toml, generated_phase4_parameters.toml / generated_phase4_scenario.toml, generated_phase5_parameters.toml / generated_phase5_scenario.toml, and generated_phase6_parameters.toml / generated_phase6_scenario.toml.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Current wiring consumes: Scenario_Controls.demand_basis plus Treatment_Duration_Assumptions for Phase 1 starts-based mode; dose_basis_default, module-specific dosing values, module FG mg per unit, module FG vialing rule, global yields, DS quantity per DP unit default, DS overage default, SS ratio, and co_pack_mode for Phase 2; active deterministic trade parameters from Trade_Inventory_FutureHooks for Phase 3; and active deterministic Phase 4 scheduling plus Phase 5 inventory controls from Trade_Inventory_FutureHooks together with the scenario-default Product_Parameters, Yield_Assumptions, and SS_Assumptions rows.</t>
+          <t xml:space="preserve">Current wiring consumes: Scenario_Controls.demand_basis plus Treatment_Duration_Assumptions for Phase 1 starts-based mode; dose_basis_default, module-specific dosing values, module FG mg per unit, module FG vialing rule, global yields, DS quantity per DP unit default, DS overage default, SS ratio, and co_pack_mode for Phase 2; active deterministic trade parameters from Trade_Inventory_FutureHooks for Phase 3; active deterministic Phase 4 scheduling plus Phase 5 inventory controls from Trade_Inventory_FutureHooks together with the scenario-default Product_Parameters, Yield_Assumptions, and SS_Assumptions rows; and active deterministic Phase 6 financial assumptions plus editable geography-bucketed Sub-Layer 1 -&gt; Sub-Layer 2 shipping/cold-chain cost parameters from Trade_Inventory_FutureHooks together with the scenario-default Product_Parameters, Yield_Assumptions, and SS_Assumptions rows.</t>
         </is>
       </c>
     </row>
@@ -272,7 +272,7 @@
       </c>
       <c r="C8" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">CML_Prevalent_Assumptions remains a dedicated artifact sheet. Populate approved pool, timing, and exhaustion metadata here without treating CML like AML/MDS segment mix logic. Trade_Inventory_FutureHooks still carries a historical name, but it now also feeds the active deterministic Phase 3 trade config plus the active Phase 4 scheduling and Phase 5 inventory config bridges.</t>
+          <t xml:space="preserve">CML_Prevalent_Assumptions remains a dedicated artifact sheet. Populate approved pool, timing, and exhaustion metadata here without treating CML like AML/MDS segment mix logic. Trade_Inventory_FutureHooks still carries a historical name, but it now also feeds the active deterministic Phase 3 trade config plus the active Phase 4 scheduling, Phase 5 inventory, and Phase 6 financial config bridges.</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:BV21"/>
+  <dimension ref="A1:CN21"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1217,6 +1217,20 @@
     <col min="71" max="71" width="18" customWidth="1"/>
     <col min="72" max="72" width="12" customWidth="1"/>
     <col min="73" max="73" width="72" customWidth="1"/>
+    <col min="74" max="74" width="18" customWidth="1"/>
+    <col min="75" max="75" width="18" customWidth="1"/>
+    <col min="76" max="76" width="18" customWidth="1"/>
+    <col min="77" max="77" width="20" customWidth="1"/>
+    <col min="78" max="78" width="18" customWidth="1"/>
+    <col min="79" max="79" width="18" customWidth="1"/>
+    <col min="80" max="80" width="18" customWidth="1"/>
+    <col min="81" max="81" width="18" customWidth="1"/>
+    <col min="82" max="82" width="18" customWidth="1"/>
+    <col min="83" max="83" width="18" customWidth="1"/>
+    <col min="84" max="84" width="18" customWidth="1"/>
+    <col min="85" max="85" width="20" customWidth="1"/>
+    <col min="86" max="86" width="18" customWidth="1"/>
+    <col min="87" max="87" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1588,6 +1602,96 @@
       <c r="BV1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_standard_cost_basis_unit</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ds_standard_cost_per_mg</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">dp_conversion_cost_per_unit</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">fg_packaging_labeling_cost_per_unit</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ss_standard_cost_per_unit</t>
+        </is>
+      </c>
+      <c r="CB1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">annual_inventory_carry_rate</t>
+        </is>
+      </c>
+      <c r="CC1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">monthly_inventory_carry_rate</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">expired_inventory_writeoff_rate</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">expired_inventory_salvage_rate</t>
+        </is>
+      </c>
+      <c r="CF1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">value_unmatched_fg_at_fg_standard_cost</t>
+        </is>
+      </c>
+      <c r="CG1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">include_trade_node_fg_value</t>
+        </is>
+      </c>
+      <c r="CH1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">use_matched_administrable_fg_value</t>
+        </is>
+      </c>
+      <c r="CI1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">phase6_enforce_unique_output_keys</t>
+        </is>
+      </c>
+      <c r="CJ1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">phase6_reconciliation_tolerance_value</t>
+        </is>
+      </c>
+      <c r="CK1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">us_fg_sub1_to_sub2_cost_per_unit</t>
+        </is>
+      </c>
+      <c r="CL1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">eu_fg_sub1_to_sub2_cost_per_unit</t>
+        </is>
+      </c>
+      <c r="CM1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">us_ss_sub1_to_sub2_cost_per_unit</t>
+        </is>
+      </c>
+      <c r="CN1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">eu_ss_sub1_to_sub2_cost_per_unit</t>
         </is>
       </c>
     </row>
@@ -1827,8 +1931,72 @@
       </c>
       <c r="BV2" t="inlineStr" s="9">
         <is>
-          <t xml:space="preserve">Active deterministic defaults for Phase 3, Phase 4, and Phase 5. Phase 5 shelf life and excess-cover values are revised placeholder baseline assumptions; edit here instead of hand-editing phase3_trade_layer.toml, phase4_production_schedule.toml, or phase5_inventory_layer.toml.</t>
-        </is>
+          <t xml:space="preserve">Active deterministic defaults for Phase 3, Phase 4, Phase 5, and Phase 6. Phase 5 shelf life/excess-cover and Phase 6 standard-cost placeholders are revised baseline assumptions; edit here instead of hand-editing phase3_trade_layer.toml, phase4_production_schedule.toml, phase5_inventory_layer.toml, or phase6_financial_layer.toml.</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">mg</t>
+        </is>
+      </c>
+      <c r="BX2" s="2">
+        <v>0.002</v>
+      </c>
+      <c r="BY2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="BZ2" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="CA2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="CB2" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="CC2" s="2">
+        <v>0.0166666666666667</v>
+      </c>
+      <c r="CD2" s="2">
+        <v>1</v>
+      </c>
+      <c r="CE2" s="2">
+        <v>0</v>
+      </c>
+      <c r="CF2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="CG2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="CH2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="CI2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="CJ2" s="2">
+        <v>1e-06</v>
+      </c>
+      <c r="CK2" s="2">
+        <v>25</v>
+      </c>
+      <c r="CL2" s="2">
+        <v>57.5</v>
+      </c>
+      <c r="CM2" s="2">
+        <v>25</v>
+      </c>
+      <c r="CN2" s="2">
+        <v>57.5</v>
       </c>
     </row>
     <row r="3">
@@ -1934,6 +2102,24 @@
           <t xml:space="preserve">Approved/sample US site activation defaults for the deterministic Phase 3 trade layer.</t>
         </is>
       </c>
+      <c r="BW3" s="2"/>
+      <c r="BX3" s="2"/>
+      <c r="BY3" s="2"/>
+      <c r="BZ3" s="2"/>
+      <c r="CA3" s="2"/>
+      <c r="CB3" s="2"/>
+      <c r="CC3" s="2"/>
+      <c r="CD3" s="2"/>
+      <c r="CE3" s="2"/>
+      <c r="CF3" s="2"/>
+      <c r="CG3" s="2"/>
+      <c r="CH3" s="2"/>
+      <c r="CI3" s="2"/>
+      <c r="CJ3" s="2"/>
+      <c r="CK3" s="2"/>
+      <c r="CL3" s="2"/>
+      <c r="CM3" s="2"/>
+      <c r="CN3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" s="3">
@@ -2038,6 +2224,24 @@
           <t xml:space="preserve">Approved/sample EU site activation defaults for the deterministic Phase 3 trade layer.</t>
         </is>
       </c>
+      <c r="BW4" s="2"/>
+      <c r="BX4" s="2"/>
+      <c r="BY4" s="2"/>
+      <c r="BZ4" s="2"/>
+      <c r="CA4" s="2"/>
+      <c r="CB4" s="2"/>
+      <c r="CC4" s="2"/>
+      <c r="CD4" s="2"/>
+      <c r="CE4" s="2"/>
+      <c r="CF4" s="2"/>
+      <c r="CG4" s="2"/>
+      <c r="CH4" s="2"/>
+      <c r="CI4" s="2"/>
+      <c r="CJ4" s="2"/>
+      <c r="CK4" s="2"/>
+      <c r="CL4" s="2"/>
+      <c r="CM4" s="2"/>
+      <c r="CN4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" s="3">
@@ -2138,6 +2342,24 @@
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
       </c>
+      <c r="BW5" s="2"/>
+      <c r="BX5" s="2"/>
+      <c r="BY5" s="2"/>
+      <c r="BZ5" s="2"/>
+      <c r="CA5" s="2"/>
+      <c r="CB5" s="2"/>
+      <c r="CC5" s="2"/>
+      <c r="CD5" s="2"/>
+      <c r="CE5" s="2"/>
+      <c r="CF5" s="2"/>
+      <c r="CG5" s="2"/>
+      <c r="CH5" s="2"/>
+      <c r="CI5" s="2"/>
+      <c r="CJ5" s="2"/>
+      <c r="CK5" s="2"/>
+      <c r="CL5" s="2"/>
+      <c r="CM5" s="2"/>
+      <c r="CN5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" s="3">
@@ -2238,6 +2460,24 @@
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
       </c>
+      <c r="BW6" s="2"/>
+      <c r="BX6" s="2"/>
+      <c r="BY6" s="2"/>
+      <c r="BZ6" s="2"/>
+      <c r="CA6" s="2"/>
+      <c r="CB6" s="2"/>
+      <c r="CC6" s="2"/>
+      <c r="CD6" s="2"/>
+      <c r="CE6" s="2"/>
+      <c r="CF6" s="2"/>
+      <c r="CG6" s="2"/>
+      <c r="CH6" s="2"/>
+      <c r="CI6" s="2"/>
+      <c r="CJ6" s="2"/>
+      <c r="CK6" s="2"/>
+      <c r="CL6" s="2"/>
+      <c r="CM6" s="2"/>
+      <c r="CN6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" s="3">
@@ -2338,6 +2578,24 @@
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
       </c>
+      <c r="BW7" s="2"/>
+      <c r="BX7" s="2"/>
+      <c r="BY7" s="2"/>
+      <c r="BZ7" s="2"/>
+      <c r="CA7" s="2"/>
+      <c r="CB7" s="2"/>
+      <c r="CC7" s="2"/>
+      <c r="CD7" s="2"/>
+      <c r="CE7" s="2"/>
+      <c r="CF7" s="2"/>
+      <c r="CG7" s="2"/>
+      <c r="CH7" s="2"/>
+      <c r="CI7" s="2"/>
+      <c r="CJ7" s="2"/>
+      <c r="CK7" s="2"/>
+      <c r="CL7" s="2"/>
+      <c r="CM7" s="2"/>
+      <c r="CN7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" s="3">
@@ -2438,6 +2696,24 @@
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
       </c>
+      <c r="BW8" s="2"/>
+      <c r="BX8" s="2"/>
+      <c r="BY8" s="2"/>
+      <c r="BZ8" s="2"/>
+      <c r="CA8" s="2"/>
+      <c r="CB8" s="2"/>
+      <c r="CC8" s="2"/>
+      <c r="CD8" s="2"/>
+      <c r="CE8" s="2"/>
+      <c r="CF8" s="2"/>
+      <c r="CG8" s="2"/>
+      <c r="CH8" s="2"/>
+      <c r="CI8" s="2"/>
+      <c r="CJ8" s="2"/>
+      <c r="CK8" s="2"/>
+      <c r="CL8" s="2"/>
+      <c r="CM8" s="2"/>
+      <c r="CN8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" s="3">
@@ -2538,6 +2814,24 @@
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
       </c>
+      <c r="BW9" s="2"/>
+      <c r="BX9" s="2"/>
+      <c r="BY9" s="2"/>
+      <c r="BZ9" s="2"/>
+      <c r="CA9" s="2"/>
+      <c r="CB9" s="2"/>
+      <c r="CC9" s="2"/>
+      <c r="CD9" s="2"/>
+      <c r="CE9" s="2"/>
+      <c r="CF9" s="2"/>
+      <c r="CG9" s="2"/>
+      <c r="CH9" s="2"/>
+      <c r="CI9" s="2"/>
+      <c r="CJ9" s="2"/>
+      <c r="CK9" s="2"/>
+      <c r="CL9" s="2"/>
+      <c r="CM9" s="2"/>
+      <c r="CN9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" s="3">
@@ -2638,6 +2932,24 @@
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
       </c>
+      <c r="BW10" s="2"/>
+      <c r="BX10" s="2"/>
+      <c r="BY10" s="2"/>
+      <c r="BZ10" s="2"/>
+      <c r="CA10" s="2"/>
+      <c r="CB10" s="2"/>
+      <c r="CC10" s="2"/>
+      <c r="CD10" s="2"/>
+      <c r="CE10" s="2"/>
+      <c r="CF10" s="2"/>
+      <c r="CG10" s="2"/>
+      <c r="CH10" s="2"/>
+      <c r="CI10" s="2"/>
+      <c r="CJ10" s="2"/>
+      <c r="CK10" s="2"/>
+      <c r="CL10" s="2"/>
+      <c r="CM10" s="2"/>
+      <c r="CN10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" s="3">
@@ -2738,6 +3050,24 @@
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
       </c>
+      <c r="BW11" s="2"/>
+      <c r="BX11" s="2"/>
+      <c r="BY11" s="2"/>
+      <c r="BZ11" s="2"/>
+      <c r="CA11" s="2"/>
+      <c r="CB11" s="2"/>
+      <c r="CC11" s="2"/>
+      <c r="CD11" s="2"/>
+      <c r="CE11" s="2"/>
+      <c r="CF11" s="2"/>
+      <c r="CG11" s="2"/>
+      <c r="CH11" s="2"/>
+      <c r="CI11" s="2"/>
+      <c r="CJ11" s="2"/>
+      <c r="CK11" s="2"/>
+      <c r="CL11" s="2"/>
+      <c r="CM11" s="2"/>
+      <c r="CN11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" s="3">
@@ -2838,6 +3168,24 @@
           <t xml:space="preserve">Approved/sample launch event.</t>
         </is>
       </c>
+      <c r="BW12" s="2"/>
+      <c r="BX12" s="2"/>
+      <c r="BY12" s="2"/>
+      <c r="BZ12" s="2"/>
+      <c r="CA12" s="2"/>
+      <c r="CB12" s="2"/>
+      <c r="CC12" s="2"/>
+      <c r="CD12" s="2"/>
+      <c r="CE12" s="2"/>
+      <c r="CF12" s="2"/>
+      <c r="CG12" s="2"/>
+      <c r="CH12" s="2"/>
+      <c r="CI12" s="2"/>
+      <c r="CJ12" s="2"/>
+      <c r="CK12" s="2"/>
+      <c r="CL12" s="2"/>
+      <c r="CM12" s="2"/>
+      <c r="CN12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" s="3"/>
@@ -2914,6 +3262,24 @@
       <c r="BT13" s="2"/>
       <c r="BU13" s="2"/>
       <c r="BV13" s="9"/>
+      <c r="BW13" s="2"/>
+      <c r="BX13" s="2"/>
+      <c r="BY13" s="2"/>
+      <c r="BZ13" s="2"/>
+      <c r="CA13" s="2"/>
+      <c r="CB13" s="2"/>
+      <c r="CC13" s="2"/>
+      <c r="CD13" s="2"/>
+      <c r="CE13" s="2"/>
+      <c r="CF13" s="2"/>
+      <c r="CG13" s="2"/>
+      <c r="CH13" s="2"/>
+      <c r="CI13" s="2"/>
+      <c r="CJ13" s="2"/>
+      <c r="CK13" s="2"/>
+      <c r="CL13" s="2"/>
+      <c r="CM13" s="2"/>
+      <c r="CN13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" s="3"/>
@@ -2990,6 +3356,24 @@
       <c r="BT14" s="2"/>
       <c r="BU14" s="2"/>
       <c r="BV14" s="9"/>
+      <c r="BW14" s="2"/>
+      <c r="BX14" s="2"/>
+      <c r="BY14" s="2"/>
+      <c r="BZ14" s="2"/>
+      <c r="CA14" s="2"/>
+      <c r="CB14" s="2"/>
+      <c r="CC14" s="2"/>
+      <c r="CD14" s="2"/>
+      <c r="CE14" s="2"/>
+      <c r="CF14" s="2"/>
+      <c r="CG14" s="2"/>
+      <c r="CH14" s="2"/>
+      <c r="CI14" s="2"/>
+      <c r="CJ14" s="2"/>
+      <c r="CK14" s="2"/>
+      <c r="CL14" s="2"/>
+      <c r="CM14" s="2"/>
+      <c r="CN14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" s="3"/>
@@ -3066,6 +3450,24 @@
       <c r="BT15" s="2"/>
       <c r="BU15" s="2"/>
       <c r="BV15" s="9"/>
+      <c r="BW15" s="2"/>
+      <c r="BX15" s="2"/>
+      <c r="BY15" s="2"/>
+      <c r="BZ15" s="2"/>
+      <c r="CA15" s="2"/>
+      <c r="CB15" s="2"/>
+      <c r="CC15" s="2"/>
+      <c r="CD15" s="2"/>
+      <c r="CE15" s="2"/>
+      <c r="CF15" s="2"/>
+      <c r="CG15" s="2"/>
+      <c r="CH15" s="2"/>
+      <c r="CI15" s="2"/>
+      <c r="CJ15" s="2"/>
+      <c r="CK15" s="2"/>
+      <c r="CL15" s="2"/>
+      <c r="CM15" s="2"/>
+      <c r="CN15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" s="3"/>
@@ -3142,6 +3544,24 @@
       <c r="BT16" s="2"/>
       <c r="BU16" s="2"/>
       <c r="BV16" s="9"/>
+      <c r="BW16" s="2"/>
+      <c r="BX16" s="2"/>
+      <c r="BY16" s="2"/>
+      <c r="BZ16" s="2"/>
+      <c r="CA16" s="2"/>
+      <c r="CB16" s="2"/>
+      <c r="CC16" s="2"/>
+      <c r="CD16" s="2"/>
+      <c r="CE16" s="2"/>
+      <c r="CF16" s="2"/>
+      <c r="CG16" s="2"/>
+      <c r="CH16" s="2"/>
+      <c r="CI16" s="2"/>
+      <c r="CJ16" s="2"/>
+      <c r="CK16" s="2"/>
+      <c r="CL16" s="2"/>
+      <c r="CM16" s="2"/>
+      <c r="CN16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" s="3"/>
@@ -3218,6 +3638,24 @@
       <c r="BT17" s="2"/>
       <c r="BU17" s="2"/>
       <c r="BV17" s="9"/>
+      <c r="BW17" s="2"/>
+      <c r="BX17" s="2"/>
+      <c r="BY17" s="2"/>
+      <c r="BZ17" s="2"/>
+      <c r="CA17" s="2"/>
+      <c r="CB17" s="2"/>
+      <c r="CC17" s="2"/>
+      <c r="CD17" s="2"/>
+      <c r="CE17" s="2"/>
+      <c r="CF17" s="2"/>
+      <c r="CG17" s="2"/>
+      <c r="CH17" s="2"/>
+      <c r="CI17" s="2"/>
+      <c r="CJ17" s="2"/>
+      <c r="CK17" s="2"/>
+      <c r="CL17" s="2"/>
+      <c r="CM17" s="2"/>
+      <c r="CN17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" s="3"/>
@@ -3294,6 +3732,24 @@
       <c r="BT18" s="2"/>
       <c r="BU18" s="2"/>
       <c r="BV18" s="9"/>
+      <c r="BW18" s="2"/>
+      <c r="BX18" s="2"/>
+      <c r="BY18" s="2"/>
+      <c r="BZ18" s="2"/>
+      <c r="CA18" s="2"/>
+      <c r="CB18" s="2"/>
+      <c r="CC18" s="2"/>
+      <c r="CD18" s="2"/>
+      <c r="CE18" s="2"/>
+      <c r="CF18" s="2"/>
+      <c r="CG18" s="2"/>
+      <c r="CH18" s="2"/>
+      <c r="CI18" s="2"/>
+      <c r="CJ18" s="2"/>
+      <c r="CK18" s="2"/>
+      <c r="CL18" s="2"/>
+      <c r="CM18" s="2"/>
+      <c r="CN18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" s="3"/>
@@ -3370,6 +3826,24 @@
       <c r="BT19" s="2"/>
       <c r="BU19" s="2"/>
       <c r="BV19" s="9"/>
+      <c r="BW19" s="2"/>
+      <c r="BX19" s="2"/>
+      <c r="BY19" s="2"/>
+      <c r="BZ19" s="2"/>
+      <c r="CA19" s="2"/>
+      <c r="CB19" s="2"/>
+      <c r="CC19" s="2"/>
+      <c r="CD19" s="2"/>
+      <c r="CE19" s="2"/>
+      <c r="CF19" s="2"/>
+      <c r="CG19" s="2"/>
+      <c r="CH19" s="2"/>
+      <c r="CI19" s="2"/>
+      <c r="CJ19" s="2"/>
+      <c r="CK19" s="2"/>
+      <c r="CL19" s="2"/>
+      <c r="CM19" s="2"/>
+      <c r="CN19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" s="3"/>
@@ -3446,6 +3920,24 @@
       <c r="BT20" s="2"/>
       <c r="BU20" s="2"/>
       <c r="BV20" s="9"/>
+      <c r="BW20" s="2"/>
+      <c r="BX20" s="2"/>
+      <c r="BY20" s="2"/>
+      <c r="BZ20" s="2"/>
+      <c r="CA20" s="2"/>
+      <c r="CB20" s="2"/>
+      <c r="CC20" s="2"/>
+      <c r="CD20" s="2"/>
+      <c r="CE20" s="2"/>
+      <c r="CF20" s="2"/>
+      <c r="CG20" s="2"/>
+      <c r="CH20" s="2"/>
+      <c r="CI20" s="2"/>
+      <c r="CJ20" s="2"/>
+      <c r="CK20" s="2"/>
+      <c r="CL20" s="2"/>
+      <c r="CM20" s="2"/>
+      <c r="CN20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" s="3"/>
@@ -3522,10 +4014,28 @@
       <c r="BT21" s="2"/>
       <c r="BU21" s="2"/>
       <c r="BV21" s="9"/>
+      <c r="BW21" s="2"/>
+      <c r="BX21" s="2"/>
+      <c r="BY21" s="2"/>
+      <c r="BZ21" s="2"/>
+      <c r="CA21" s="2"/>
+      <c r="CB21" s="2"/>
+      <c r="CC21" s="2"/>
+      <c r="CD21" s="2"/>
+      <c r="CE21" s="2"/>
+      <c r="CF21" s="2"/>
+      <c r="CG21" s="2"/>
+      <c r="CH21" s="2"/>
+      <c r="CI21" s="2"/>
+      <c r="CJ21" s="2"/>
+      <c r="CK21" s="2"/>
+      <c r="CL21" s="2"/>
+      <c r="CM21" s="2"/>
+      <c r="CN21" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BV1"/>
-  <dataValidations count="6">
+  <autoFilter ref="A1:CJ1"/>
+  <dataValidations count="7">
     <dataValidation type="list" sqref="B2:B21" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$O$2:$O$4</formula1>
     </dataValidation>
@@ -3543,6 +4053,9 @@
     </dataValidation>
     <dataValidation type="list" sqref="BU2:BU21" showErrorMessage="1" allowBlank="1">
       <formula1>Lookup_Lists!$J$2:$J$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="CF2:CI21" showErrorMessage="1" allowBlank="1">
+      <formula1>Lookup_Lists!$F$2:$F$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>